<commit_message>
fix(cap.2): logica de cimentacion completa - excavacion 0.60, sub-base 0.30, zapatas agregadas (concreto+acero), solado bajo zapatas
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
@@ -25,6 +25,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.7.1" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4.8.1" sheetId="18" state="visible" r:id="rId18"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5.2.1" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.2.3 ZAPATAS" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2.3.2 ACERO ZAPATAS" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -2296,28 +2298,58 @@
       <c r="A19" s="8" t="n"/>
       <c r="B19" s="29" t="n"/>
       <c r="J19" s="30" t="n"/>
-      <c r="K19" s="20" t="n"/>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>Solado bajo zapatas Z-1 (2.30x2.30)</t>
+        </is>
+      </c>
       <c r="L19" s="21" t="n"/>
       <c r="M19" s="22" t="n"/>
-      <c r="N19" s="18" t="n"/>
-      <c r="O19" s="18" t="n"/>
-      <c r="P19" s="18" t="n"/>
-      <c r="Q19" s="18" t="n"/>
-      <c r="R19" s="18" t="n"/>
+      <c r="N19" s="18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="O19" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="Q19" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R19" s="18">
+        <f>N19*O19*P19*Q19</f>
+        <v/>
+      </c>
       <c r="S19" s="9" t="n"/>
     </row>
     <row r="20" ht="15.6" customHeight="1" s="24">
       <c r="A20" s="8" t="n"/>
       <c r="B20" s="29" t="n"/>
       <c r="J20" s="30" t="n"/>
-      <c r="K20" s="20" t="n"/>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>Solado bajo zapatas Z-2 (2.15x2.15)</t>
+        </is>
+      </c>
       <c r="L20" s="21" t="n"/>
       <c r="M20" s="22" t="n"/>
-      <c r="N20" s="18" t="n"/>
-      <c r="O20" s="18" t="n"/>
-      <c r="P20" s="18" t="n"/>
-      <c r="Q20" s="18" t="n"/>
-      <c r="R20" s="18" t="n"/>
+      <c r="N20" s="18" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="O20" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" s="18" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="Q20" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R20" s="18">
+        <f>N20*O20*P20*Q20</f>
+        <v/>
+      </c>
       <c r="S20" s="9" t="n"/>
     </row>
     <row r="21" ht="15.6" customHeight="1" s="24">
@@ -2620,7 +2652,11 @@
     </row>
     <row r="40" ht="15.6" customHeight="1" s="24">
       <c r="A40" s="8" t="n"/>
-      <c r="B40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>AGREGADO: solado de limpieza e=0.05 tambien bajo las 8 zapatas (el detalle de zapata lo muestra). Medido por m2.</t>
+        </is>
+      </c>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="27" t="n"/>
       <c r="E40" s="27" t="n"/>
@@ -14171,6 +14207,2258 @@
     <mergeCell ref="K20:M20"/>
     <mergeCell ref="K21:M21"/>
     <mergeCell ref="B52:D52"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="K26:M26"/>
+    <mergeCell ref="K29:M29"/>
+    <mergeCell ref="P6:R6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.42578125" customWidth="1" style="24" min="13" max="13"/>
+    <col width="11.5703125" bestFit="1" customWidth="1" style="24" min="14" max="14"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" style="24" min="15" max="15"/>
+    <col width="11.140625" bestFit="1" customWidth="1" style="24" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.6" customHeight="1" s="24">
+      <c r="A1" s="5" t="n"/>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
+      <c r="E1" s="38" t="n"/>
+      <c r="F1" s="38" t="n"/>
+      <c r="G1" s="38" t="n"/>
+      <c r="H1" s="38" t="n"/>
+      <c r="I1" s="38" t="n"/>
+      <c r="J1" s="38" t="n"/>
+      <c r="K1" s="38" t="n"/>
+      <c r="L1" s="38" t="n"/>
+      <c r="M1" s="38" t="n"/>
+      <c r="N1" s="38" t="n"/>
+      <c r="O1" s="38" t="n"/>
+      <c r="P1" s="38" t="n"/>
+      <c r="Q1" s="38" t="n"/>
+      <c r="R1" s="38" t="n"/>
+      <c r="S1" s="7" t="n"/>
+    </row>
+    <row r="2" ht="15.6" customHeight="1" s="24">
+      <c r="A2" s="8" t="n"/>
+      <c r="B2" s="23" t="n"/>
+      <c r="C2" s="23" t="n"/>
+      <c r="D2" s="23" t="n"/>
+      <c r="E2" s="23" t="n"/>
+      <c r="F2" s="23" t="n"/>
+      <c r="G2" s="23" t="n"/>
+      <c r="H2" s="23" t="n"/>
+      <c r="I2" s="23" t="n"/>
+      <c r="J2" s="23" t="n"/>
+      <c r="K2" s="23" t="n"/>
+      <c r="L2" s="23" t="n"/>
+      <c r="M2" s="23" t="n"/>
+      <c r="N2" s="23" t="n"/>
+      <c r="O2" s="23" t="n"/>
+      <c r="P2" s="23" t="n"/>
+      <c r="Q2" s="23" t="n"/>
+      <c r="R2" s="23" t="n"/>
+      <c r="S2" s="9" t="n"/>
+    </row>
+    <row r="3" ht="15.6" customHeight="1" s="24">
+      <c r="A3" s="8" t="n"/>
+      <c r="B3" s="20" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="28" t="n"/>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>MEMORIA DE CÁLCULO</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="27" t="n"/>
+      <c r="K3" s="27" t="n"/>
+      <c r="L3" s="27" t="n"/>
+      <c r="M3" s="27" t="n"/>
+      <c r="N3" s="27" t="n"/>
+      <c r="O3" s="28" t="n"/>
+      <c r="P3" s="25" t="inlineStr">
+        <is>
+          <t>CONTRATO No.</t>
+        </is>
+      </c>
+      <c r="Q3" s="21" t="n"/>
+      <c r="R3" s="22" t="n"/>
+      <c r="S3" s="9" t="n"/>
+    </row>
+    <row r="4" ht="15.6" customHeight="1" s="24">
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="29" t="n"/>
+      <c r="D4" s="30" t="n"/>
+      <c r="E4" s="29" t="n"/>
+      <c r="O4" s="30" t="n"/>
+      <c r="P4" s="34" t="n"/>
+      <c r="Q4" s="21" t="n"/>
+      <c r="R4" s="22" t="n"/>
+      <c r="S4" s="9" t="n"/>
+    </row>
+    <row r="5" ht="15.6" customHeight="1" s="24">
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="29" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="29" t="n"/>
+      <c r="O5" s="30" t="n"/>
+      <c r="P5" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CORTE No. </t>
+        </is>
+      </c>
+      <c r="Q5" s="21" t="n"/>
+      <c r="R5" s="22" t="n"/>
+      <c r="S5" s="9" t="n"/>
+    </row>
+    <row r="6" ht="15.6" customHeight="1" s="24">
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="29" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="29" t="n"/>
+      <c r="O6" s="30" t="n"/>
+      <c r="P6" s="34" t="n"/>
+      <c r="Q6" s="21" t="n"/>
+      <c r="R6" s="22" t="n"/>
+      <c r="S6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="15.6" customHeight="1" s="24">
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="29" t="n"/>
+      <c r="D7" s="30" t="n"/>
+      <c r="E7" s="31" t="n"/>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
+      <c r="H7" s="32" t="n"/>
+      <c r="I7" s="32" t="n"/>
+      <c r="J7" s="32" t="n"/>
+      <c r="K7" s="32" t="n"/>
+      <c r="L7" s="32" t="n"/>
+      <c r="M7" s="32" t="n"/>
+      <c r="N7" s="32" t="n"/>
+      <c r="O7" s="33" t="n"/>
+      <c r="P7" s="25" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="Q7" s="25" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="R7" s="25" t="inlineStr">
+        <is>
+          <t>AAAA</t>
+        </is>
+      </c>
+      <c r="S7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="15.6" customHeight="1" s="24">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="29" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>PROYECTO: MÓDULO 1 COLEGIO</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="27" t="n"/>
+      <c r="I8" s="27" t="n"/>
+      <c r="J8" s="27" t="n"/>
+      <c r="K8" s="27" t="n"/>
+      <c r="L8" s="27" t="n"/>
+      <c r="M8" s="27" t="n"/>
+      <c r="N8" s="27" t="n"/>
+      <c r="O8" s="28" t="n"/>
+      <c r="P8" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q8" s="20" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="R8" s="20" t="n">
+        <v>2025</v>
+      </c>
+      <c r="S8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="15.6" customHeight="1" s="24">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="29" t="n"/>
+      <c r="D9" s="30" t="n"/>
+      <c r="E9" s="29" t="n"/>
+      <c r="O9" s="30" t="n"/>
+      <c r="P9" s="25" t="inlineStr">
+        <is>
+          <t>PÁGINA</t>
+        </is>
+      </c>
+      <c r="Q9" s="28" t="n"/>
+      <c r="R9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="9" t="n"/>
+    </row>
+    <row r="10" ht="15.6" customHeight="1" s="24">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="n"/>
+      <c r="H10" s="32" t="n"/>
+      <c r="I10" s="32" t="n"/>
+      <c r="J10" s="32" t="n"/>
+      <c r="K10" s="32" t="n"/>
+      <c r="L10" s="32" t="n"/>
+      <c r="M10" s="32" t="n"/>
+      <c r="N10" s="32" t="n"/>
+      <c r="O10" s="33" t="n"/>
+      <c r="P10" s="31" t="n"/>
+      <c r="Q10" s="33" t="n"/>
+      <c r="R10" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="15.6" customHeight="1" s="24">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="23" t="n"/>
+      <c r="S11" s="9" t="n"/>
+    </row>
+    <row r="12" ht="15.6" customHeight="1" s="24">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>CONTRATISTA</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="20" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="21" t="n"/>
+      <c r="I12" s="21" t="n"/>
+      <c r="J12" s="21" t="n"/>
+      <c r="K12" s="21" t="n"/>
+      <c r="L12" s="21" t="n"/>
+      <c r="M12" s="22" t="n"/>
+      <c r="N12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NIT No. </t>
+        </is>
+      </c>
+      <c r="O12" s="22" t="n"/>
+      <c r="P12" s="20" t="n"/>
+      <c r="Q12" s="21" t="n"/>
+      <c r="R12" s="22" t="n"/>
+      <c r="S12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="15.6" customHeight="1" s="24">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>CAPÍTULO</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>CIMENTACION</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="22" t="n"/>
+      <c r="I13" s="25" t="inlineStr">
+        <is>
+          <t>ITEM</t>
+        </is>
+      </c>
+      <c r="J13" s="20" t="inlineStr">
+        <is>
+          <t>2.2.3</t>
+        </is>
+      </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>Zapatas concreto 3000psi</t>
+        </is>
+      </c>
+      <c r="L13" s="21" t="n"/>
+      <c r="M13" s="21" t="n"/>
+      <c r="N13" s="21" t="n"/>
+      <c r="O13" s="21" t="n"/>
+      <c r="P13" s="22" t="n"/>
+      <c r="Q13" s="25" t="inlineStr">
+        <is>
+          <t>U/MED</t>
+        </is>
+      </c>
+      <c r="R13" s="20" t="inlineStr">
+        <is>
+          <t>M3</t>
+        </is>
+      </c>
+      <c r="S13" s="9" t="n"/>
+    </row>
+    <row r="14" ht="15.6" customHeight="1" s="24">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="23" t="n"/>
+      <c r="S14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="15.6" customHeight="1" s="24">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>IMAGEN/REFERENCIA</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="22" t="n"/>
+      <c r="K15" s="25" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="L15" s="27" t="n"/>
+      <c r="M15" s="28" t="n"/>
+      <c r="N15" s="25" t="inlineStr">
+        <is>
+          <t>Dimensiones</t>
+        </is>
+      </c>
+      <c r="O15" s="21" t="n"/>
+      <c r="P15" s="22" t="n"/>
+      <c r="Q15" s="25" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R15" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="S15" s="9" t="n"/>
+    </row>
+    <row r="16" ht="15.6" customHeight="1" s="24">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="27" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="28" t="n"/>
+      <c r="K16" s="31" t="n"/>
+      <c r="L16" s="32" t="n"/>
+      <c r="M16" s="33" t="n"/>
+      <c r="N16" s="25" t="inlineStr">
+        <is>
+          <t>Ancho (m)</t>
+        </is>
+      </c>
+      <c r="O16" s="25" t="inlineStr">
+        <is>
+          <t>Alto (m)</t>
+        </is>
+      </c>
+      <c r="P16" s="25" t="inlineStr">
+        <is>
+          <t>Largo (m)</t>
+        </is>
+      </c>
+      <c r="Q16" s="26" t="n"/>
+      <c r="R16" s="26" t="n"/>
+      <c r="S16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="15.6" customHeight="1" s="24">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="29" t="n"/>
+      <c r="J17" s="30" t="n"/>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>Zapatas Z-1 (2.30x2.30x0.40) - ejes 2A,3A,2B,3B</t>
+        </is>
+      </c>
+      <c r="L17" s="21" t="n"/>
+      <c r="M17" s="22" t="n"/>
+      <c r="N17" s="18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="O17" s="18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P17" s="18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="Q17" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R17" s="18">
+        <f>N17*O17*P17*Q17</f>
+        <v/>
+      </c>
+      <c r="S17" s="9" t="n"/>
+    </row>
+    <row r="18" ht="15.6" customHeight="1" s="24">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="29" t="n"/>
+      <c r="J18" s="30" t="n"/>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>Zapatas Z-2 (2.15x2.15x0.40) - ejes 1A,4A,1B,4B</t>
+        </is>
+      </c>
+      <c r="L18" s="21" t="n"/>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="18" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="O18" s="18" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P18" s="18" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="Q18" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R18" s="18">
+        <f>N18*O18*P18*Q18</f>
+        <v/>
+      </c>
+      <c r="S18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="15.6" customHeight="1" s="24">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="29" t="n"/>
+      <c r="J19" s="30" t="n"/>
+      <c r="K19" s="20" t="n"/>
+      <c r="L19" s="21" t="n"/>
+      <c r="M19" s="22" t="n"/>
+      <c r="N19" s="18" t="n"/>
+      <c r="O19" s="18" t="n"/>
+      <c r="P19" s="18" t="n"/>
+      <c r="Q19" s="18" t="n"/>
+      <c r="R19" s="18" t="n"/>
+      <c r="S19" s="9" t="n"/>
+    </row>
+    <row r="20" ht="15.6" customHeight="1" s="24">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="29" t="n"/>
+      <c r="J20" s="30" t="n"/>
+      <c r="K20" s="20" t="n"/>
+      <c r="L20" s="21" t="n"/>
+      <c r="M20" s="22" t="n"/>
+      <c r="N20" s="18" t="n"/>
+      <c r="O20" s="18" t="n"/>
+      <c r="P20" s="18" t="n"/>
+      <c r="Q20" s="18" t="n"/>
+      <c r="R20" s="18" t="n"/>
+      <c r="S20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="15.6" customHeight="1" s="24">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="29" t="n"/>
+      <c r="J21" s="30" t="n"/>
+      <c r="K21" s="20" t="n"/>
+      <c r="L21" s="21" t="n"/>
+      <c r="M21" s="22" t="n"/>
+      <c r="N21" s="18" t="n"/>
+      <c r="O21" s="18" t="n"/>
+      <c r="P21" s="18" t="n"/>
+      <c r="Q21" s="18" t="n"/>
+      <c r="R21" s="18" t="n"/>
+      <c r="S21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="15.6" customHeight="1" s="24">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="29" t="n"/>
+      <c r="J22" s="30" t="n"/>
+      <c r="K22" s="20" t="n"/>
+      <c r="L22" s="21" t="n"/>
+      <c r="M22" s="22" t="n"/>
+      <c r="N22" s="18" t="n"/>
+      <c r="O22" s="18" t="n"/>
+      <c r="P22" s="18" t="n"/>
+      <c r="Q22" s="18" t="n"/>
+      <c r="R22" s="18" t="n"/>
+      <c r="S22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="15.6" customHeight="1" s="24">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="29" t="n"/>
+      <c r="J23" s="30" t="n"/>
+      <c r="K23" s="20" t="n"/>
+      <c r="L23" s="21" t="n"/>
+      <c r="M23" s="22" t="n"/>
+      <c r="N23" s="18" t="n"/>
+      <c r="O23" s="18" t="n"/>
+      <c r="P23" s="18" t="n"/>
+      <c r="Q23" s="18" t="n"/>
+      <c r="R23" s="18" t="n"/>
+      <c r="S23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="15.6" customHeight="1" s="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="29" t="n"/>
+      <c r="J24" s="30" t="n"/>
+      <c r="K24" s="20" t="n"/>
+      <c r="L24" s="21" t="n"/>
+      <c r="M24" s="22" t="n"/>
+      <c r="N24" s="18" t="n"/>
+      <c r="O24" s="18" t="n"/>
+      <c r="P24" s="18" t="n"/>
+      <c r="Q24" s="18" t="n"/>
+      <c r="R24" s="18" t="n"/>
+      <c r="S24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="15.6" customHeight="1" s="24">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="29" t="n"/>
+      <c r="J25" s="30" t="n"/>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="21" t="n"/>
+      <c r="M25" s="22" t="n"/>
+      <c r="N25" s="18" t="n"/>
+      <c r="O25" s="18" t="n"/>
+      <c r="P25" s="18" t="n"/>
+      <c r="Q25" s="18" t="n"/>
+      <c r="R25" s="18" t="n"/>
+      <c r="S25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="15.6" customHeight="1" s="24">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="29" t="n"/>
+      <c r="J26" s="30" t="n"/>
+      <c r="K26" s="20" t="n"/>
+      <c r="L26" s="21" t="n"/>
+      <c r="M26" s="22" t="n"/>
+      <c r="N26" s="18" t="n"/>
+      <c r="O26" s="18" t="n"/>
+      <c r="P26" s="18" t="n"/>
+      <c r="Q26" s="18" t="n"/>
+      <c r="R26" s="18" t="n"/>
+      <c r="S26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="15.6" customHeight="1" s="24">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="29" t="n"/>
+      <c r="J27" s="30" t="n"/>
+      <c r="K27" s="20" t="n"/>
+      <c r="L27" s="21" t="n"/>
+      <c r="M27" s="22" t="n"/>
+      <c r="N27" s="18" t="n"/>
+      <c r="O27" s="18" t="n"/>
+      <c r="P27" s="18" t="n"/>
+      <c r="Q27" s="18" t="n"/>
+      <c r="R27" s="18" t="n"/>
+      <c r="S27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="15.6" customHeight="1" s="24">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="29" t="n"/>
+      <c r="J28" s="30" t="n"/>
+      <c r="K28" s="20" t="n"/>
+      <c r="L28" s="21" t="n"/>
+      <c r="M28" s="22" t="n"/>
+      <c r="N28" s="18" t="n"/>
+      <c r="O28" s="18" t="n"/>
+      <c r="P28" s="18" t="n"/>
+      <c r="Q28" s="18" t="n"/>
+      <c r="R28" s="18" t="n"/>
+      <c r="S28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="15.6" customHeight="1" s="24">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="29" t="n"/>
+      <c r="J29" s="30" t="n"/>
+      <c r="K29" s="20" t="n"/>
+      <c r="L29" s="21" t="n"/>
+      <c r="M29" s="22" t="n"/>
+      <c r="N29" s="18" t="n"/>
+      <c r="O29" s="18" t="n"/>
+      <c r="P29" s="18" t="n"/>
+      <c r="Q29" s="18" t="n"/>
+      <c r="R29" s="18" t="n"/>
+      <c r="S29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="15.6" customHeight="1" s="24">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="29" t="n"/>
+      <c r="J30" s="30" t="n"/>
+      <c r="K30" s="20" t="n"/>
+      <c r="L30" s="21" t="n"/>
+      <c r="M30" s="22" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="18" t="n"/>
+      <c r="P30" s="18" t="n"/>
+      <c r="Q30" s="18" t="n"/>
+      <c r="R30" s="18" t="n"/>
+      <c r="S30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="15.6" customHeight="1" s="24">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="29" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="20" t="n"/>
+      <c r="L31" s="21" t="n"/>
+      <c r="M31" s="22" t="n"/>
+      <c r="N31" s="18" t="n"/>
+      <c r="O31" s="18" t="n"/>
+      <c r="P31" s="18" t="n"/>
+      <c r="Q31" s="18" t="n"/>
+      <c r="R31" s="18" t="n"/>
+      <c r="S31" s="9" t="n"/>
+    </row>
+    <row r="32" ht="15.6" customHeight="1" s="24">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="29" t="n"/>
+      <c r="J32" s="30" t="n"/>
+      <c r="K32" s="20" t="n"/>
+      <c r="L32" s="21" t="n"/>
+      <c r="M32" s="22" t="n"/>
+      <c r="N32" s="18" t="n"/>
+      <c r="O32" s="18" t="n"/>
+      <c r="P32" s="18" t="n"/>
+      <c r="Q32" s="18" t="n"/>
+      <c r="R32" s="18" t="n"/>
+      <c r="S32" s="9" t="n"/>
+    </row>
+    <row r="33" ht="15.6" customHeight="1" s="24">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="29" t="n"/>
+      <c r="J33" s="30" t="n"/>
+      <c r="K33" s="20" t="n"/>
+      <c r="L33" s="21" t="n"/>
+      <c r="M33" s="22" t="n"/>
+      <c r="N33" s="18" t="n"/>
+      <c r="O33" s="18" t="n"/>
+      <c r="P33" s="18" t="n"/>
+      <c r="Q33" s="18" t="n"/>
+      <c r="R33" s="18" t="n"/>
+      <c r="S33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="15.6" customHeight="1" s="24">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="29" t="n"/>
+      <c r="J34" s="30" t="n"/>
+      <c r="K34" s="20" t="n"/>
+      <c r="L34" s="21" t="n"/>
+      <c r="M34" s="22" t="n"/>
+      <c r="N34" s="18" t="n"/>
+      <c r="O34" s="18" t="n"/>
+      <c r="P34" s="18" t="n"/>
+      <c r="Q34" s="18" t="n"/>
+      <c r="R34" s="18" t="n"/>
+      <c r="S34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="15.6" customHeight="1" s="24">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="29" t="n"/>
+      <c r="J35" s="30" t="n"/>
+      <c r="K35" s="20" t="n"/>
+      <c r="L35" s="21" t="n"/>
+      <c r="M35" s="22" t="n"/>
+      <c r="N35" s="18" t="n"/>
+      <c r="O35" s="18" t="n"/>
+      <c r="P35" s="18" t="n"/>
+      <c r="Q35" s="18" t="n"/>
+      <c r="R35" s="18" t="n"/>
+      <c r="S35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="15.6" customHeight="1" s="24">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="29" t="n"/>
+      <c r="J36" s="30" t="n"/>
+      <c r="K36" s="20" t="n"/>
+      <c r="L36" s="21" t="n"/>
+      <c r="M36" s="22" t="n"/>
+      <c r="N36" s="18" t="n"/>
+      <c r="O36" s="18" t="n"/>
+      <c r="P36" s="18" t="n"/>
+      <c r="Q36" s="18" t="n"/>
+      <c r="R36" s="18" t="n"/>
+      <c r="S36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="15.6" customHeight="1" s="24">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="31" t="n"/>
+      <c r="C37" s="32" t="n"/>
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="32" t="n"/>
+      <c r="F37" s="32" t="n"/>
+      <c r="G37" s="32" t="n"/>
+      <c r="H37" s="32" t="n"/>
+      <c r="I37" s="32" t="n"/>
+      <c r="J37" s="33" t="n"/>
+      <c r="K37" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L37" s="21" t="n"/>
+      <c r="M37" s="21" t="n"/>
+      <c r="N37" s="21" t="n"/>
+      <c r="O37" s="21" t="n"/>
+      <c r="P37" s="21" t="n"/>
+      <c r="Q37" s="22" t="n"/>
+      <c r="R37" s="19">
+        <f>SUM(R17:R36)</f>
+        <v/>
+      </c>
+      <c r="S37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="15.6" customHeight="1" s="24">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="23" t="n"/>
+      <c r="C38" s="23" t="n"/>
+      <c r="D38" s="23" t="n"/>
+      <c r="E38" s="23" t="n"/>
+      <c r="F38" s="23" t="n"/>
+      <c r="G38" s="23" t="n"/>
+      <c r="H38" s="23" t="n"/>
+      <c r="I38" s="23" t="n"/>
+      <c r="J38" s="23" t="n"/>
+      <c r="K38" s="13" t="n"/>
+      <c r="L38" s="13" t="n"/>
+      <c r="M38" s="13" t="n"/>
+      <c r="N38" s="13" t="n"/>
+      <c r="O38" s="13" t="n"/>
+      <c r="P38" s="13" t="n"/>
+      <c r="Q38" s="13" t="n"/>
+      <c r="R38" s="13" t="n"/>
+      <c r="S38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="15.6" customHeight="1" s="24">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="25" t="inlineStr">
+        <is>
+          <t>OBSERVACIONES</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="n"/>
+      <c r="D39" s="21" t="n"/>
+      <c r="E39" s="21" t="n"/>
+      <c r="F39" s="21" t="n"/>
+      <c r="G39" s="21" t="n"/>
+      <c r="H39" s="21" t="n"/>
+      <c r="I39" s="21" t="n"/>
+      <c r="J39" s="21" t="n"/>
+      <c r="K39" s="21" t="n"/>
+      <c r="L39" s="21" t="n"/>
+      <c r="M39" s="21" t="n"/>
+      <c r="N39" s="21" t="n"/>
+      <c r="O39" s="21" t="n"/>
+      <c r="P39" s="21" t="n"/>
+      <c r="Q39" s="21" t="n"/>
+      <c r="R39" s="22" t="n"/>
+      <c r="S39" s="9" t="n"/>
+    </row>
+    <row r="40" ht="15.6" customHeight="1" s="24">
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>AGREGADO: 8 zapatas (4 Z-1 + 4 Z-2), H=0.40. Falta la linea correspondiente en el presupuesto (2.2.3). Concreto 3000 psi.</t>
+        </is>
+      </c>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="27" t="n"/>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="27" t="n"/>
+      <c r="H40" s="27" t="n"/>
+      <c r="I40" s="27" t="n"/>
+      <c r="J40" s="27" t="n"/>
+      <c r="K40" s="27" t="n"/>
+      <c r="L40" s="27" t="n"/>
+      <c r="M40" s="27" t="n"/>
+      <c r="N40" s="27" t="n"/>
+      <c r="O40" s="27" t="n"/>
+      <c r="P40" s="27" t="n"/>
+      <c r="Q40" s="27" t="n"/>
+      <c r="R40" s="28" t="n"/>
+      <c r="S40" s="9" t="n"/>
+    </row>
+    <row r="41" ht="15.6" customHeight="1" s="24">
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="29" t="n"/>
+      <c r="R41" s="30" t="n"/>
+      <c r="S41" s="9" t="n"/>
+    </row>
+    <row r="42" ht="15.6" customHeight="1" s="24">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="29" t="n"/>
+      <c r="R42" s="30" t="n"/>
+      <c r="S42" s="9" t="n"/>
+    </row>
+    <row r="43" ht="15.6" customHeight="1" s="24">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="29" t="n"/>
+      <c r="R43" s="30" t="n"/>
+      <c r="S43" s="9" t="n"/>
+    </row>
+    <row r="44" ht="15.6" customHeight="1" s="24">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="31" t="n"/>
+      <c r="C44" s="32" t="n"/>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="32" t="n"/>
+      <c r="F44" s="32" t="n"/>
+      <c r="G44" s="32" t="n"/>
+      <c r="H44" s="32" t="n"/>
+      <c r="I44" s="32" t="n"/>
+      <c r="J44" s="32" t="n"/>
+      <c r="K44" s="32" t="n"/>
+      <c r="L44" s="32" t="n"/>
+      <c r="M44" s="32" t="n"/>
+      <c r="N44" s="32" t="n"/>
+      <c r="O44" s="32" t="n"/>
+      <c r="P44" s="32" t="n"/>
+      <c r="Q44" s="32" t="n"/>
+      <c r="R44" s="33" t="n"/>
+      <c r="S44" s="9" t="n"/>
+    </row>
+    <row r="45" ht="15.6" customHeight="1" s="24">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="23" t="n"/>
+      <c r="C45" s="23" t="n"/>
+      <c r="D45" s="23" t="n"/>
+      <c r="E45" s="23" t="n"/>
+      <c r="F45" s="23" t="n"/>
+      <c r="G45" s="23" t="n"/>
+      <c r="H45" s="23" t="n"/>
+      <c r="I45" s="23" t="n"/>
+      <c r="J45" s="23" t="n"/>
+      <c r="K45" s="23" t="n"/>
+      <c r="L45" s="23" t="n"/>
+      <c r="M45" s="23" t="n"/>
+      <c r="N45" s="23" t="n"/>
+      <c r="O45" s="23" t="n"/>
+      <c r="P45" s="23" t="n"/>
+      <c r="Q45" s="23" t="n"/>
+      <c r="R45" s="23" t="n"/>
+      <c r="S45" s="9" t="n"/>
+    </row>
+    <row r="46" ht="15.6" customHeight="1" s="24">
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="23" t="n"/>
+      <c r="C46" s="23" t="n"/>
+      <c r="D46" s="23" t="n"/>
+      <c r="E46" s="23" t="n"/>
+      <c r="F46" s="23" t="n"/>
+      <c r="G46" s="23" t="n"/>
+      <c r="H46" s="23" t="n"/>
+      <c r="I46" s="23" t="n"/>
+      <c r="J46" s="23" t="n"/>
+      <c r="K46" s="23" t="n"/>
+      <c r="L46" s="23" t="n"/>
+      <c r="M46" s="23" t="n"/>
+      <c r="N46" s="23" t="n"/>
+      <c r="O46" s="23" t="n"/>
+      <c r="P46" s="23" t="n"/>
+      <c r="Q46" s="23" t="n"/>
+      <c r="R46" s="23" t="n"/>
+      <c r="S46" s="9" t="n"/>
+    </row>
+    <row r="47" ht="15.6" customHeight="1" s="24">
+      <c r="A47" s="14" t="n"/>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>Elaboró</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="n"/>
+      <c r="D47" s="16" t="n"/>
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="16" t="n"/>
+      <c r="G47" s="16" t="n"/>
+      <c r="H47" s="16" t="n"/>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>Revisó</t>
+        </is>
+      </c>
+      <c r="J47" s="16" t="n"/>
+      <c r="K47" s="16" t="n"/>
+      <c r="L47" s="16" t="n"/>
+      <c r="M47" s="16" t="n"/>
+      <c r="N47" s="16" t="n"/>
+      <c r="O47" s="16" t="n"/>
+      <c r="P47" s="15" t="inlineStr">
+        <is>
+          <t>Aprobó</t>
+        </is>
+      </c>
+      <c r="Q47" s="16" t="n"/>
+      <c r="R47" s="16" t="n"/>
+      <c r="S47" s="17" t="n"/>
+    </row>
+    <row r="48" ht="15.6" customHeight="1" s="24">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="23" t="n"/>
+      <c r="C48" s="23" t="n"/>
+      <c r="D48" s="23" t="n"/>
+      <c r="E48" s="23" t="n"/>
+      <c r="F48" s="23" t="n"/>
+      <c r="G48" s="23" t="n"/>
+      <c r="H48" s="23" t="n"/>
+      <c r="I48" s="23" t="n"/>
+      <c r="J48" s="23" t="n"/>
+      <c r="K48" s="23" t="n"/>
+      <c r="L48" s="23" t="n"/>
+      <c r="M48" s="23" t="n"/>
+      <c r="N48" s="23" t="n"/>
+      <c r="O48" s="23" t="n"/>
+      <c r="P48" s="23" t="n"/>
+      <c r="Q48" s="23" t="n"/>
+      <c r="R48" s="23" t="n"/>
+      <c r="S48" s="9" t="n"/>
+    </row>
+    <row r="49" ht="15.6" customHeight="1" s="24">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="23" t="n"/>
+      <c r="C49" s="23" t="n"/>
+      <c r="D49" s="23" t="n"/>
+      <c r="E49" s="23" t="n"/>
+      <c r="F49" s="23" t="n"/>
+      <c r="G49" s="23" t="n"/>
+      <c r="H49" s="23" t="n"/>
+      <c r="I49" s="23" t="n"/>
+      <c r="J49" s="23" t="n"/>
+      <c r="K49" s="23" t="n"/>
+      <c r="L49" s="23" t="n"/>
+      <c r="M49" s="23" t="n"/>
+      <c r="N49" s="23" t="n"/>
+      <c r="O49" s="23" t="n"/>
+      <c r="P49" s="23" t="n"/>
+      <c r="Q49" s="23" t="n"/>
+      <c r="R49" s="23" t="n"/>
+      <c r="S49" s="9" t="n"/>
+    </row>
+    <row r="50" ht="15.6" customHeight="1" s="24">
+      <c r="A50" s="8" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="11" t="n"/>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="23" t="n"/>
+      <c r="F50" s="23" t="n"/>
+      <c r="G50" s="23" t="n"/>
+      <c r="H50" s="23" t="n"/>
+      <c r="I50" s="11" t="n"/>
+      <c r="J50" s="11" t="n"/>
+      <c r="K50" s="11" t="n"/>
+      <c r="L50" s="23" t="n"/>
+      <c r="M50" s="23" t="n"/>
+      <c r="N50" s="23" t="n"/>
+      <c r="O50" s="23" t="n"/>
+      <c r="P50" s="11" t="n"/>
+      <c r="Q50" s="11" t="n"/>
+      <c r="R50" s="11" t="n"/>
+      <c r="S50" s="9" t="n"/>
+    </row>
+    <row r="51" ht="15.6" customHeight="1" s="24">
+      <c r="A51" s="8" t="n"/>
+      <c r="E51" s="23" t="n"/>
+      <c r="F51" s="23" t="n"/>
+      <c r="G51" s="23" t="n"/>
+      <c r="H51" s="23" t="n"/>
+      <c r="I51" s="38" t="n"/>
+      <c r="J51" s="27" t="n"/>
+      <c r="K51" s="27" t="n"/>
+      <c r="L51" s="23" t="n"/>
+      <c r="M51" s="23" t="n"/>
+      <c r="N51" s="23" t="n"/>
+      <c r="O51" s="23" t="n"/>
+      <c r="P51" s="38" t="n"/>
+      <c r="Q51" s="27" t="n"/>
+      <c r="R51" s="27" t="n"/>
+      <c r="S51" s="9" t="n"/>
+    </row>
+    <row r="52" ht="15.6" customHeight="1" s="24">
+      <c r="A52" s="8" t="n"/>
+      <c r="E52" s="23" t="n"/>
+      <c r="F52" s="23" t="n"/>
+      <c r="G52" s="23" t="n"/>
+      <c r="H52" s="23" t="n"/>
+      <c r="I52" s="23" t="n"/>
+      <c r="L52" s="23" t="n"/>
+      <c r="M52" s="23" t="n"/>
+      <c r="N52" s="23" t="n"/>
+      <c r="O52" s="23" t="n"/>
+      <c r="P52" s="23" t="n"/>
+      <c r="S52" s="9" t="n"/>
+    </row>
+    <row r="53" ht="15.6" customHeight="1" s="24">
+      <c r="A53" s="8" t="n"/>
+      <c r="E53" s="23" t="n"/>
+      <c r="F53" s="23" t="n"/>
+      <c r="G53" s="23" t="n"/>
+      <c r="H53" s="23" t="n"/>
+      <c r="I53" s="36" t="n"/>
+      <c r="L53" s="23" t="n"/>
+      <c r="M53" s="23" t="n"/>
+      <c r="N53" s="23" t="n"/>
+      <c r="O53" s="23" t="n"/>
+      <c r="P53" s="36" t="n"/>
+      <c r="S53" s="9" t="n"/>
+    </row>
+    <row r="54" ht="15.6" customHeight="1" s="24">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="23" t="n"/>
+      <c r="C54" s="23" t="n"/>
+      <c r="D54" s="23" t="n"/>
+      <c r="E54" s="23" t="n"/>
+      <c r="F54" s="23" t="n"/>
+      <c r="G54" s="23" t="n"/>
+      <c r="H54" s="23" t="n"/>
+      <c r="I54" s="23" t="n"/>
+      <c r="J54" s="23" t="n"/>
+      <c r="K54" s="23" t="n"/>
+      <c r="L54" s="23" t="n"/>
+      <c r="M54" s="23" t="n"/>
+      <c r="N54" s="23" t="n"/>
+      <c r="O54" s="23" t="n"/>
+      <c r="P54" s="23" t="n"/>
+      <c r="Q54" s="23" t="n"/>
+      <c r="R54" s="23" t="n"/>
+      <c r="S54" s="9" t="n"/>
+    </row>
+    <row r="55" ht="15.6" customHeight="1" s="24">
+      <c r="A55" s="10" t="n"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="11" t="n"/>
+      <c r="H55" s="11" t="n"/>
+      <c r="I55" s="11" t="n"/>
+      <c r="J55" s="11" t="n"/>
+      <c r="K55" s="11" t="n"/>
+      <c r="L55" s="11" t="n"/>
+      <c r="M55" s="11" t="n"/>
+      <c r="N55" s="11" t="n"/>
+      <c r="O55" s="11" t="n"/>
+      <c r="P55" s="11" t="n"/>
+      <c r="Q55" s="11" t="n"/>
+      <c r="R55" s="11" t="n"/>
+      <c r="S55" s="12" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="51">
+    <mergeCell ref="B40:R44"/>
+    <mergeCell ref="P52:R52"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="D12:M12"/>
+    <mergeCell ref="K22:M22"/>
+    <mergeCell ref="E3:O7"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="K31:M31"/>
+    <mergeCell ref="R15:R16"/>
+    <mergeCell ref="B16:J37"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="K15:M16"/>
+    <mergeCell ref="K37:Q37"/>
+    <mergeCell ref="E8:O10"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="B39:R39"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="K23:M23"/>
+    <mergeCell ref="P53:R53"/>
+    <mergeCell ref="B11:R11"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="Q15:Q16"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="B14:R14"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="B3:D10"/>
+    <mergeCell ref="K28:M28"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="K13:P13"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="P51:R51"/>
+    <mergeCell ref="K30:M30"/>
+    <mergeCell ref="K25:M25"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="K24:M24"/>
+    <mergeCell ref="P9:Q10"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="K21:M21"/>
+    <mergeCell ref="K35:M35"/>
+    <mergeCell ref="K26:M26"/>
+    <mergeCell ref="K29:M29"/>
+    <mergeCell ref="P6:R6"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:S55"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col width="11.42578125" customWidth="1" style="24" min="13" max="13"/>
+    <col width="11.5703125" bestFit="1" customWidth="1" style="24" min="14" max="14"/>
+    <col width="9.42578125" bestFit="1" customWidth="1" style="24" min="15" max="15"/>
+    <col width="11.140625" bestFit="1" customWidth="1" style="24" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="15.6" customHeight="1" s="24">
+      <c r="A1" s="5" t="n"/>
+      <c r="B1" s="38" t="n"/>
+      <c r="C1" s="38" t="n"/>
+      <c r="D1" s="38" t="n"/>
+      <c r="E1" s="38" t="n"/>
+      <c r="F1" s="38" t="n"/>
+      <c r="G1" s="38" t="n"/>
+      <c r="H1" s="38" t="n"/>
+      <c r="I1" s="38" t="n"/>
+      <c r="J1" s="38" t="n"/>
+      <c r="K1" s="38" t="n"/>
+      <c r="L1" s="38" t="n"/>
+      <c r="M1" s="38" t="n"/>
+      <c r="N1" s="38" t="n"/>
+      <c r="O1" s="38" t="n"/>
+      <c r="P1" s="38" t="n"/>
+      <c r="Q1" s="38" t="n"/>
+      <c r="R1" s="38" t="n"/>
+      <c r="S1" s="7" t="n"/>
+    </row>
+    <row r="2" ht="15.6" customHeight="1" s="24">
+      <c r="A2" s="8" t="n"/>
+      <c r="B2" s="23" t="n"/>
+      <c r="C2" s="23" t="n"/>
+      <c r="D2" s="23" t="n"/>
+      <c r="E2" s="23" t="n"/>
+      <c r="F2" s="23" t="n"/>
+      <c r="G2" s="23" t="n"/>
+      <c r="H2" s="23" t="n"/>
+      <c r="I2" s="23" t="n"/>
+      <c r="J2" s="23" t="n"/>
+      <c r="K2" s="23" t="n"/>
+      <c r="L2" s="23" t="n"/>
+      <c r="M2" s="23" t="n"/>
+      <c r="N2" s="23" t="n"/>
+      <c r="O2" s="23" t="n"/>
+      <c r="P2" s="23" t="n"/>
+      <c r="Q2" s="23" t="n"/>
+      <c r="R2" s="23" t="n"/>
+      <c r="S2" s="9" t="n"/>
+    </row>
+    <row r="3" ht="15.6" customHeight="1" s="24">
+      <c r="A3" s="8" t="n"/>
+      <c r="B3" s="20" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="28" t="n"/>
+      <c r="E3" s="35" t="inlineStr">
+        <is>
+          <t>MEMORIA DE CÁLCULO</t>
+        </is>
+      </c>
+      <c r="F3" s="27" t="n"/>
+      <c r="G3" s="27" t="n"/>
+      <c r="H3" s="27" t="n"/>
+      <c r="I3" s="27" t="n"/>
+      <c r="J3" s="27" t="n"/>
+      <c r="K3" s="27" t="n"/>
+      <c r="L3" s="27" t="n"/>
+      <c r="M3" s="27" t="n"/>
+      <c r="N3" s="27" t="n"/>
+      <c r="O3" s="28" t="n"/>
+      <c r="P3" s="25" t="inlineStr">
+        <is>
+          <t>CONTRATO No.</t>
+        </is>
+      </c>
+      <c r="Q3" s="21" t="n"/>
+      <c r="R3" s="22" t="n"/>
+      <c r="S3" s="9" t="n"/>
+    </row>
+    <row r="4" ht="15.6" customHeight="1" s="24">
+      <c r="A4" s="8" t="n"/>
+      <c r="B4" s="29" t="n"/>
+      <c r="D4" s="30" t="n"/>
+      <c r="E4" s="29" t="n"/>
+      <c r="O4" s="30" t="n"/>
+      <c r="P4" s="34" t="n"/>
+      <c r="Q4" s="21" t="n"/>
+      <c r="R4" s="22" t="n"/>
+      <c r="S4" s="9" t="n"/>
+    </row>
+    <row r="5" ht="15.6" customHeight="1" s="24">
+      <c r="A5" s="8" t="n"/>
+      <c r="B5" s="29" t="n"/>
+      <c r="D5" s="30" t="n"/>
+      <c r="E5" s="29" t="n"/>
+      <c r="O5" s="30" t="n"/>
+      <c r="P5" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">CORTE No. </t>
+        </is>
+      </c>
+      <c r="Q5" s="21" t="n"/>
+      <c r="R5" s="22" t="n"/>
+      <c r="S5" s="9" t="n"/>
+    </row>
+    <row r="6" ht="15.6" customHeight="1" s="24">
+      <c r="A6" s="8" t="n"/>
+      <c r="B6" s="29" t="n"/>
+      <c r="D6" s="30" t="n"/>
+      <c r="E6" s="29" t="n"/>
+      <c r="O6" s="30" t="n"/>
+      <c r="P6" s="34" t="n"/>
+      <c r="Q6" s="21" t="n"/>
+      <c r="R6" s="22" t="n"/>
+      <c r="S6" s="9" t="n"/>
+    </row>
+    <row r="7" ht="15.6" customHeight="1" s="24">
+      <c r="A7" s="8" t="n"/>
+      <c r="B7" s="29" t="n"/>
+      <c r="D7" s="30" t="n"/>
+      <c r="E7" s="31" t="n"/>
+      <c r="F7" s="32" t="n"/>
+      <c r="G7" s="32" t="n"/>
+      <c r="H7" s="32" t="n"/>
+      <c r="I7" s="32" t="n"/>
+      <c r="J7" s="32" t="n"/>
+      <c r="K7" s="32" t="n"/>
+      <c r="L7" s="32" t="n"/>
+      <c r="M7" s="32" t="n"/>
+      <c r="N7" s="32" t="n"/>
+      <c r="O7" s="33" t="n"/>
+      <c r="P7" s="25" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="Q7" s="25" t="inlineStr">
+        <is>
+          <t>MMM</t>
+        </is>
+      </c>
+      <c r="R7" s="25" t="inlineStr">
+        <is>
+          <t>AAAA</t>
+        </is>
+      </c>
+      <c r="S7" s="9" t="n"/>
+    </row>
+    <row r="8" ht="15.6" customHeight="1" s="24">
+      <c r="A8" s="8" t="n"/>
+      <c r="B8" s="29" t="n"/>
+      <c r="D8" s="30" t="n"/>
+      <c r="E8" s="37" t="inlineStr">
+        <is>
+          <t>PROYECTO: MÓDULO 1 COLEGIO</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n"/>
+      <c r="G8" s="27" t="n"/>
+      <c r="H8" s="27" t="n"/>
+      <c r="I8" s="27" t="n"/>
+      <c r="J8" s="27" t="n"/>
+      <c r="K8" s="27" t="n"/>
+      <c r="L8" s="27" t="n"/>
+      <c r="M8" s="27" t="n"/>
+      <c r="N8" s="27" t="n"/>
+      <c r="O8" s="28" t="n"/>
+      <c r="P8" s="20" t="n">
+        <v>30</v>
+      </c>
+      <c r="Q8" s="20" t="inlineStr">
+        <is>
+          <t>SEP</t>
+        </is>
+      </c>
+      <c r="R8" s="20" t="n">
+        <v>2025</v>
+      </c>
+      <c r="S8" s="9" t="n"/>
+    </row>
+    <row r="9" ht="15.6" customHeight="1" s="24">
+      <c r="A9" s="8" t="n"/>
+      <c r="B9" s="29" t="n"/>
+      <c r="D9" s="30" t="n"/>
+      <c r="E9" s="29" t="n"/>
+      <c r="O9" s="30" t="n"/>
+      <c r="P9" s="25" t="inlineStr">
+        <is>
+          <t>PÁGINA</t>
+        </is>
+      </c>
+      <c r="Q9" s="28" t="n"/>
+      <c r="R9" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S9" s="9" t="n"/>
+    </row>
+    <row r="10" ht="15.6" customHeight="1" s="24">
+      <c r="A10" s="8" t="n"/>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="31" t="n"/>
+      <c r="F10" s="32" t="n"/>
+      <c r="G10" s="32" t="n"/>
+      <c r="H10" s="32" t="n"/>
+      <c r="I10" s="32" t="n"/>
+      <c r="J10" s="32" t="n"/>
+      <c r="K10" s="32" t="n"/>
+      <c r="L10" s="32" t="n"/>
+      <c r="M10" s="32" t="n"/>
+      <c r="N10" s="32" t="n"/>
+      <c r="O10" s="33" t="n"/>
+      <c r="P10" s="31" t="n"/>
+      <c r="Q10" s="33" t="n"/>
+      <c r="R10" s="34" t="n">
+        <v>1</v>
+      </c>
+      <c r="S10" s="9" t="n"/>
+    </row>
+    <row r="11" ht="15.6" customHeight="1" s="24">
+      <c r="A11" s="8" t="n"/>
+      <c r="B11" s="23" t="n"/>
+      <c r="S11" s="9" t="n"/>
+    </row>
+    <row r="12" ht="15.6" customHeight="1" s="24">
+      <c r="A12" s="8" t="n"/>
+      <c r="B12" s="25" t="inlineStr">
+        <is>
+          <t>CONTRATISTA</t>
+        </is>
+      </c>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="20" t="n"/>
+      <c r="E12" s="21" t="n"/>
+      <c r="F12" s="21" t="n"/>
+      <c r="G12" s="21" t="n"/>
+      <c r="H12" s="21" t="n"/>
+      <c r="I12" s="21" t="n"/>
+      <c r="J12" s="21" t="n"/>
+      <c r="K12" s="21" t="n"/>
+      <c r="L12" s="21" t="n"/>
+      <c r="M12" s="22" t="n"/>
+      <c r="N12" s="25" t="inlineStr">
+        <is>
+          <t xml:space="preserve">NIT No. </t>
+        </is>
+      </c>
+      <c r="O12" s="22" t="n"/>
+      <c r="P12" s="20" t="n"/>
+      <c r="Q12" s="21" t="n"/>
+      <c r="R12" s="22" t="n"/>
+      <c r="S12" s="9" t="n"/>
+    </row>
+    <row r="13" ht="15.6" customHeight="1" s="24">
+      <c r="A13" s="8" t="n"/>
+      <c r="B13" s="25" t="inlineStr">
+        <is>
+          <t>CAPÍTULO</t>
+        </is>
+      </c>
+      <c r="C13" s="20" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D13" s="20" t="inlineStr">
+        <is>
+          <t>REFUERZOS / ACERO</t>
+        </is>
+      </c>
+      <c r="E13" s="21" t="n"/>
+      <c r="F13" s="21" t="n"/>
+      <c r="G13" s="21" t="n"/>
+      <c r="H13" s="22" t="n"/>
+      <c r="I13" s="25" t="inlineStr">
+        <is>
+          <t>ITEM</t>
+        </is>
+      </c>
+      <c r="J13" s="20" t="inlineStr">
+        <is>
+          <t>2.3.2</t>
+        </is>
+      </c>
+      <c r="K13" s="20" t="inlineStr">
+        <is>
+          <t>Acero figurado zapatas</t>
+        </is>
+      </c>
+      <c r="L13" s="21" t="n"/>
+      <c r="M13" s="21" t="n"/>
+      <c r="N13" s="21" t="n"/>
+      <c r="O13" s="21" t="n"/>
+      <c r="P13" s="22" t="n"/>
+      <c r="Q13" s="25" t="inlineStr">
+        <is>
+          <t>U/MED</t>
+        </is>
+      </c>
+      <c r="R13" s="20" t="inlineStr">
+        <is>
+          <t>KG</t>
+        </is>
+      </c>
+      <c r="S13" s="9" t="n"/>
+    </row>
+    <row r="14" ht="15.6" customHeight="1" s="24">
+      <c r="A14" s="8" t="n"/>
+      <c r="B14" s="23" t="n"/>
+      <c r="S14" s="9" t="n"/>
+    </row>
+    <row r="15" ht="15.6" customHeight="1" s="24">
+      <c r="A15" s="8" t="n"/>
+      <c r="B15" s="25" t="inlineStr">
+        <is>
+          <t>IMAGEN/REFERENCIA</t>
+        </is>
+      </c>
+      <c r="C15" s="21" t="n"/>
+      <c r="D15" s="21" t="n"/>
+      <c r="E15" s="21" t="n"/>
+      <c r="F15" s="21" t="n"/>
+      <c r="G15" s="21" t="n"/>
+      <c r="H15" s="21" t="n"/>
+      <c r="I15" s="21" t="n"/>
+      <c r="J15" s="22" t="n"/>
+      <c r="K15" s="25" t="inlineStr">
+        <is>
+          <t>Descripción</t>
+        </is>
+      </c>
+      <c r="L15" s="27" t="n"/>
+      <c r="M15" s="28" t="n"/>
+      <c r="N15" s="25" t="inlineStr">
+        <is>
+          <t>Dimensiones</t>
+        </is>
+      </c>
+      <c r="O15" s="21" t="n"/>
+      <c r="P15" s="22" t="n"/>
+      <c r="Q15" s="25" t="inlineStr">
+        <is>
+          <t>Cantidad</t>
+        </is>
+      </c>
+      <c r="R15" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="S15" s="9" t="n"/>
+    </row>
+    <row r="16" ht="15.6" customHeight="1" s="24">
+      <c r="A16" s="8" t="n"/>
+      <c r="B16" s="20" t="n"/>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="27" t="n"/>
+      <c r="E16" s="27" t="n"/>
+      <c r="F16" s="27" t="n"/>
+      <c r="G16" s="27" t="n"/>
+      <c r="H16" s="27" t="n"/>
+      <c r="I16" s="27" t="n"/>
+      <c r="J16" s="28" t="n"/>
+      <c r="K16" s="31" t="n"/>
+      <c r="L16" s="32" t="n"/>
+      <c r="M16" s="33" t="n"/>
+      <c r="N16" s="25" t="inlineStr">
+        <is>
+          <t>Ancho (m)</t>
+        </is>
+      </c>
+      <c r="O16" s="25" t="inlineStr">
+        <is>
+          <t>Alto (m)</t>
+        </is>
+      </c>
+      <c r="P16" s="25" t="inlineStr">
+        <is>
+          <t>Largo (m)</t>
+        </is>
+      </c>
+      <c r="Q16" s="26" t="n"/>
+      <c r="R16" s="26" t="n"/>
+      <c r="S16" s="9" t="n"/>
+    </row>
+    <row r="17" ht="15.6" customHeight="1" s="24">
+      <c r="A17" s="8" t="n"/>
+      <c r="B17" s="29" t="n"/>
+      <c r="J17" s="30" t="n"/>
+      <c r="K17" s="20" t="inlineStr">
+        <is>
+          <t>Z-1: 4 zap, #5@0.20 dos sentidos (est.)</t>
+        </is>
+      </c>
+      <c r="L17" s="21" t="n"/>
+      <c r="M17" s="22" t="n"/>
+      <c r="N17" s="18" t="n">
+        <v>9.85</v>
+      </c>
+      <c r="O17" s="18" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="P17" s="18" t="n">
+        <v>21.95</v>
+      </c>
+      <c r="Q17" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="R17" s="18" t="n">
+        <v>327.8</v>
+      </c>
+      <c r="S17" s="9" t="n"/>
+    </row>
+    <row r="18" ht="15.6" customHeight="1" s="24">
+      <c r="A18" s="8" t="n"/>
+      <c r="B18" s="29" t="n"/>
+      <c r="J18" s="30" t="n"/>
+      <c r="K18" s="20" t="inlineStr">
+        <is>
+          <t>Z-2: 4 zap, #5@0.20 dos sentidos (est.)</t>
+        </is>
+      </c>
+      <c r="L18" s="21" t="n"/>
+      <c r="M18" s="22" t="n"/>
+      <c r="N18" s="18" t="n"/>
+      <c r="O18" s="18" t="n"/>
+      <c r="P18" s="18" t="n"/>
+      <c r="Q18" s="18" t="n"/>
+      <c r="R18" s="18" t="n">
+        <v>280</v>
+      </c>
+      <c r="S18" s="9" t="n"/>
+    </row>
+    <row r="19" ht="15.6" customHeight="1" s="24">
+      <c r="A19" s="8" t="n"/>
+      <c r="B19" s="29" t="n"/>
+      <c r="J19" s="30" t="n"/>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>Subtotal (kg)</t>
+        </is>
+      </c>
+      <c r="L19" s="21" t="n"/>
+      <c r="M19" s="22" t="n"/>
+      <c r="N19" s="18" t="n"/>
+      <c r="O19" s="18" t="n"/>
+      <c r="P19" s="18" t="n"/>
+      <c r="Q19" s="18" t="n"/>
+      <c r="R19" s="18" t="n">
+        <v>607.8</v>
+      </c>
+      <c r="S19" s="9" t="n"/>
+    </row>
+    <row r="20" ht="15.6" customHeight="1" s="24">
+      <c r="A20" s="8" t="n"/>
+      <c r="B20" s="29" t="n"/>
+      <c r="J20" s="30" t="n"/>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>Con 10% desperd/traslapo (kg)</t>
+        </is>
+      </c>
+      <c r="L20" s="21" t="n"/>
+      <c r="M20" s="22" t="n"/>
+      <c r="N20" s="18" t="n"/>
+      <c r="O20" s="18" t="n"/>
+      <c r="P20" s="18" t="n"/>
+      <c r="Q20" s="18" t="n"/>
+      <c r="R20" s="18" t="n">
+        <v>668.6</v>
+      </c>
+      <c r="S20" s="9" t="n"/>
+    </row>
+    <row r="21" ht="15.6" customHeight="1" s="24">
+      <c r="A21" s="8" t="n"/>
+      <c r="B21" s="29" t="n"/>
+      <c r="J21" s="30" t="n"/>
+      <c r="K21" s="20" t="n"/>
+      <c r="L21" s="21" t="n"/>
+      <c r="M21" s="22" t="n"/>
+      <c r="N21" s="18" t="n"/>
+      <c r="O21" s="18" t="n"/>
+      <c r="P21" s="18" t="n"/>
+      <c r="Q21" s="18" t="n"/>
+      <c r="R21" s="18" t="n"/>
+      <c r="S21" s="9" t="n"/>
+    </row>
+    <row r="22" ht="15.6" customHeight="1" s="24">
+      <c r="A22" s="8" t="n"/>
+      <c r="B22" s="29" t="n"/>
+      <c r="J22" s="30" t="n"/>
+      <c r="K22" s="20" t="n"/>
+      <c r="L22" s="21" t="n"/>
+      <c r="M22" s="22" t="n"/>
+      <c r="N22" s="18" t="n"/>
+      <c r="O22" s="18" t="n"/>
+      <c r="P22" s="18" t="n"/>
+      <c r="Q22" s="18" t="n"/>
+      <c r="R22" s="18" t="n"/>
+      <c r="S22" s="9" t="n"/>
+    </row>
+    <row r="23" ht="15.6" customHeight="1" s="24">
+      <c r="A23" s="8" t="n"/>
+      <c r="B23" s="29" t="n"/>
+      <c r="J23" s="30" t="n"/>
+      <c r="K23" s="20" t="n"/>
+      <c r="L23" s="21" t="n"/>
+      <c r="M23" s="22" t="n"/>
+      <c r="N23" s="18" t="n"/>
+      <c r="O23" s="18" t="n"/>
+      <c r="P23" s="18" t="n"/>
+      <c r="Q23" s="18" t="n"/>
+      <c r="R23" s="18" t="n"/>
+      <c r="S23" s="9" t="n"/>
+    </row>
+    <row r="24" ht="15.6" customHeight="1" s="24">
+      <c r="A24" s="8" t="n"/>
+      <c r="B24" s="29" t="n"/>
+      <c r="J24" s="30" t="n"/>
+      <c r="K24" s="20" t="n"/>
+      <c r="L24" s="21" t="n"/>
+      <c r="M24" s="22" t="n"/>
+      <c r="N24" s="18" t="n"/>
+      <c r="O24" s="18" t="n"/>
+      <c r="P24" s="18" t="n"/>
+      <c r="Q24" s="18" t="n"/>
+      <c r="R24" s="18" t="n"/>
+      <c r="S24" s="9" t="n"/>
+    </row>
+    <row r="25" ht="15.6" customHeight="1" s="24">
+      <c r="A25" s="8" t="n"/>
+      <c r="B25" s="29" t="n"/>
+      <c r="J25" s="30" t="n"/>
+      <c r="K25" s="20" t="n"/>
+      <c r="L25" s="21" t="n"/>
+      <c r="M25" s="22" t="n"/>
+      <c r="N25" s="18" t="n"/>
+      <c r="O25" s="18" t="n"/>
+      <c r="P25" s="18" t="n"/>
+      <c r="Q25" s="18" t="n"/>
+      <c r="R25" s="18" t="n"/>
+      <c r="S25" s="9" t="n"/>
+    </row>
+    <row r="26" ht="15.6" customHeight="1" s="24">
+      <c r="A26" s="8" t="n"/>
+      <c r="B26" s="29" t="n"/>
+      <c r="J26" s="30" t="n"/>
+      <c r="K26" s="20" t="n"/>
+      <c r="L26" s="21" t="n"/>
+      <c r="M26" s="22" t="n"/>
+      <c r="N26" s="18" t="n"/>
+      <c r="O26" s="18" t="n"/>
+      <c r="P26" s="18" t="n"/>
+      <c r="Q26" s="18" t="n"/>
+      <c r="R26" s="18" t="n"/>
+      <c r="S26" s="9" t="n"/>
+    </row>
+    <row r="27" ht="15.6" customHeight="1" s="24">
+      <c r="A27" s="8" t="n"/>
+      <c r="B27" s="29" t="n"/>
+      <c r="J27" s="30" t="n"/>
+      <c r="K27" s="20" t="n"/>
+      <c r="L27" s="21" t="n"/>
+      <c r="M27" s="22" t="n"/>
+      <c r="N27" s="18" t="n"/>
+      <c r="O27" s="18" t="n"/>
+      <c r="P27" s="18" t="n"/>
+      <c r="Q27" s="18" t="n"/>
+      <c r="R27" s="18" t="n"/>
+      <c r="S27" s="9" t="n"/>
+    </row>
+    <row r="28" ht="15.6" customHeight="1" s="24">
+      <c r="A28" s="8" t="n"/>
+      <c r="B28" s="29" t="n"/>
+      <c r="J28" s="30" t="n"/>
+      <c r="K28" s="20" t="n"/>
+      <c r="L28" s="21" t="n"/>
+      <c r="M28" s="22" t="n"/>
+      <c r="N28" s="18" t="n"/>
+      <c r="O28" s="18" t="n"/>
+      <c r="P28" s="18" t="n"/>
+      <c r="Q28" s="18" t="n"/>
+      <c r="R28" s="18" t="n"/>
+      <c r="S28" s="9" t="n"/>
+    </row>
+    <row r="29" ht="15.6" customHeight="1" s="24">
+      <c r="A29" s="8" t="n"/>
+      <c r="B29" s="29" t="n"/>
+      <c r="J29" s="30" t="n"/>
+      <c r="K29" s="20" t="n"/>
+      <c r="L29" s="21" t="n"/>
+      <c r="M29" s="22" t="n"/>
+      <c r="N29" s="18" t="n"/>
+      <c r="O29" s="18" t="n"/>
+      <c r="P29" s="18" t="n"/>
+      <c r="Q29" s="18" t="n"/>
+      <c r="R29" s="18" t="n"/>
+      <c r="S29" s="9" t="n"/>
+    </row>
+    <row r="30" ht="15.6" customHeight="1" s="24">
+      <c r="A30" s="8" t="n"/>
+      <c r="B30" s="29" t="n"/>
+      <c r="J30" s="30" t="n"/>
+      <c r="K30" s="20" t="n"/>
+      <c r="L30" s="21" t="n"/>
+      <c r="M30" s="22" t="n"/>
+      <c r="N30" s="18" t="n"/>
+      <c r="O30" s="18" t="n"/>
+      <c r="P30" s="18" t="n"/>
+      <c r="Q30" s="18" t="n"/>
+      <c r="R30" s="18" t="n"/>
+      <c r="S30" s="9" t="n"/>
+    </row>
+    <row r="31" ht="15.6" customHeight="1" s="24">
+      <c r="A31" s="8" t="n"/>
+      <c r="B31" s="29" t="n"/>
+      <c r="J31" s="30" t="n"/>
+      <c r="K31" s="20" t="n"/>
+      <c r="L31" s="21" t="n"/>
+      <c r="M31" s="22" t="n"/>
+      <c r="N31" s="18" t="n"/>
+      <c r="O31" s="18" t="n"/>
+      <c r="P31" s="18" t="n"/>
+      <c r="Q31" s="18" t="n"/>
+      <c r="R31" s="18" t="n"/>
+      <c r="S31" s="9" t="n"/>
+    </row>
+    <row r="32" ht="15.6" customHeight="1" s="24">
+      <c r="A32" s="8" t="n"/>
+      <c r="B32" s="29" t="n"/>
+      <c r="J32" s="30" t="n"/>
+      <c r="K32" s="20" t="n"/>
+      <c r="L32" s="21" t="n"/>
+      <c r="M32" s="22" t="n"/>
+      <c r="N32" s="18" t="n"/>
+      <c r="O32" s="18" t="n"/>
+      <c r="P32" s="18" t="n"/>
+      <c r="Q32" s="18" t="n"/>
+      <c r="R32" s="18" t="n"/>
+      <c r="S32" s="9" t="n"/>
+    </row>
+    <row r="33" ht="15.6" customHeight="1" s="24">
+      <c r="A33" s="8" t="n"/>
+      <c r="B33" s="29" t="n"/>
+      <c r="J33" s="30" t="n"/>
+      <c r="K33" s="20" t="n"/>
+      <c r="L33" s="21" t="n"/>
+      <c r="M33" s="22" t="n"/>
+      <c r="N33" s="18" t="n"/>
+      <c r="O33" s="18" t="n"/>
+      <c r="P33" s="18" t="n"/>
+      <c r="Q33" s="18" t="n"/>
+      <c r="R33" s="18" t="n"/>
+      <c r="S33" s="9" t="n"/>
+    </row>
+    <row r="34" ht="15.6" customHeight="1" s="24">
+      <c r="A34" s="8" t="n"/>
+      <c r="B34" s="29" t="n"/>
+      <c r="J34" s="30" t="n"/>
+      <c r="K34" s="20" t="n"/>
+      <c r="L34" s="21" t="n"/>
+      <c r="M34" s="22" t="n"/>
+      <c r="N34" s="18" t="n"/>
+      <c r="O34" s="18" t="n"/>
+      <c r="P34" s="18" t="n"/>
+      <c r="Q34" s="18" t="n"/>
+      <c r="R34" s="18" t="n"/>
+      <c r="S34" s="9" t="n"/>
+    </row>
+    <row r="35" ht="15.6" customHeight="1" s="24">
+      <c r="A35" s="8" t="n"/>
+      <c r="B35" s="29" t="n"/>
+      <c r="J35" s="30" t="n"/>
+      <c r="K35" s="20" t="n"/>
+      <c r="L35" s="21" t="n"/>
+      <c r="M35" s="22" t="n"/>
+      <c r="N35" s="18" t="n"/>
+      <c r="O35" s="18" t="n"/>
+      <c r="P35" s="18" t="n"/>
+      <c r="Q35" s="18" t="n"/>
+      <c r="R35" s="18" t="n"/>
+      <c r="S35" s="9" t="n"/>
+    </row>
+    <row r="36" ht="15.6" customHeight="1" s="24">
+      <c r="A36" s="8" t="n"/>
+      <c r="B36" s="29" t="n"/>
+      <c r="J36" s="30" t="n"/>
+      <c r="K36" s="20" t="n"/>
+      <c r="L36" s="21" t="n"/>
+      <c r="M36" s="22" t="n"/>
+      <c r="N36" s="18" t="n"/>
+      <c r="O36" s="18" t="n"/>
+      <c r="P36" s="18" t="n"/>
+      <c r="Q36" s="18" t="n"/>
+      <c r="R36" s="18" t="n"/>
+      <c r="S36" s="9" t="n"/>
+    </row>
+    <row r="37" ht="15.6" customHeight="1" s="24">
+      <c r="A37" s="8" t="n"/>
+      <c r="B37" s="31" t="n"/>
+      <c r="C37" s="32" t="n"/>
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="32" t="n"/>
+      <c r="F37" s="32" t="n"/>
+      <c r="G37" s="32" t="n"/>
+      <c r="H37" s="32" t="n"/>
+      <c r="I37" s="32" t="n"/>
+      <c r="J37" s="33" t="n"/>
+      <c r="K37" s="25" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="L37" s="21" t="n"/>
+      <c r="M37" s="21" t="n"/>
+      <c r="N37" s="21" t="n"/>
+      <c r="O37" s="21" t="n"/>
+      <c r="P37" s="21" t="n"/>
+      <c r="Q37" s="22" t="n"/>
+      <c r="R37" s="19">
+        <f>R20</f>
+        <v/>
+      </c>
+      <c r="S37" s="9" t="n"/>
+    </row>
+    <row r="38" ht="15.6" customHeight="1" s="24">
+      <c r="A38" s="8" t="n"/>
+      <c r="B38" s="23" t="n"/>
+      <c r="C38" s="23" t="n"/>
+      <c r="D38" s="23" t="n"/>
+      <c r="E38" s="23" t="n"/>
+      <c r="F38" s="23" t="n"/>
+      <c r="G38" s="23" t="n"/>
+      <c r="H38" s="23" t="n"/>
+      <c r="I38" s="23" t="n"/>
+      <c r="J38" s="23" t="n"/>
+      <c r="K38" s="13" t="n"/>
+      <c r="L38" s="13" t="n"/>
+      <c r="M38" s="13" t="n"/>
+      <c r="N38" s="13" t="n"/>
+      <c r="O38" s="13" t="n"/>
+      <c r="P38" s="13" t="n"/>
+      <c r="Q38" s="13" t="n"/>
+      <c r="R38" s="13" t="n"/>
+      <c r="S38" s="9" t="n"/>
+    </row>
+    <row r="39" ht="15.6" customHeight="1" s="24">
+      <c r="A39" s="8" t="n"/>
+      <c r="B39" s="25" t="inlineStr">
+        <is>
+          <t>OBSERVACIONES</t>
+        </is>
+      </c>
+      <c r="C39" s="21" t="n"/>
+      <c r="D39" s="21" t="n"/>
+      <c r="E39" s="21" t="n"/>
+      <c r="F39" s="21" t="n"/>
+      <c r="G39" s="21" t="n"/>
+      <c r="H39" s="21" t="n"/>
+      <c r="I39" s="21" t="n"/>
+      <c r="J39" s="21" t="n"/>
+      <c r="K39" s="21" t="n"/>
+      <c r="L39" s="21" t="n"/>
+      <c r="M39" s="21" t="n"/>
+      <c r="N39" s="21" t="n"/>
+      <c r="O39" s="21" t="n"/>
+      <c r="P39" s="21" t="n"/>
+      <c r="Q39" s="21" t="n"/>
+      <c r="R39" s="22" t="n"/>
+      <c r="S39" s="9" t="n"/>
+    </row>
+    <row r="40" ht="15.6" customHeight="1" s="24">
+      <c r="A40" s="8" t="n"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>AGREGADO (ESTIMACION): #5 @0.20 en ambos sentidos, ambas zapatas. El peso exacto debe salir de la cartilla de hierros (DLNET). Falta linea en el presupuesto.</t>
+        </is>
+      </c>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="27" t="n"/>
+      <c r="F40" s="27" t="n"/>
+      <c r="G40" s="27" t="n"/>
+      <c r="H40" s="27" t="n"/>
+      <c r="I40" s="27" t="n"/>
+      <c r="J40" s="27" t="n"/>
+      <c r="K40" s="27" t="n"/>
+      <c r="L40" s="27" t="n"/>
+      <c r="M40" s="27" t="n"/>
+      <c r="N40" s="27" t="n"/>
+      <c r="O40" s="27" t="n"/>
+      <c r="P40" s="27" t="n"/>
+      <c r="Q40" s="27" t="n"/>
+      <c r="R40" s="28" t="n"/>
+      <c r="S40" s="9" t="n"/>
+    </row>
+    <row r="41" ht="15.6" customHeight="1" s="24">
+      <c r="A41" s="8" t="n"/>
+      <c r="B41" s="29" t="n"/>
+      <c r="R41" s="30" t="n"/>
+      <c r="S41" s="9" t="n"/>
+    </row>
+    <row r="42" ht="15.6" customHeight="1" s="24">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="29" t="n"/>
+      <c r="R42" s="30" t="n"/>
+      <c r="S42" s="9" t="n"/>
+    </row>
+    <row r="43" ht="15.6" customHeight="1" s="24">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="29" t="n"/>
+      <c r="R43" s="30" t="n"/>
+      <c r="S43" s="9" t="n"/>
+    </row>
+    <row r="44" ht="15.6" customHeight="1" s="24">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="31" t="n"/>
+      <c r="C44" s="32" t="n"/>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="32" t="n"/>
+      <c r="F44" s="32" t="n"/>
+      <c r="G44" s="32" t="n"/>
+      <c r="H44" s="32" t="n"/>
+      <c r="I44" s="32" t="n"/>
+      <c r="J44" s="32" t="n"/>
+      <c r="K44" s="32" t="n"/>
+      <c r="L44" s="32" t="n"/>
+      <c r="M44" s="32" t="n"/>
+      <c r="N44" s="32" t="n"/>
+      <c r="O44" s="32" t="n"/>
+      <c r="P44" s="32" t="n"/>
+      <c r="Q44" s="32" t="n"/>
+      <c r="R44" s="33" t="n"/>
+      <c r="S44" s="9" t="n"/>
+    </row>
+    <row r="45" ht="15.6" customHeight="1" s="24">
+      <c r="A45" s="8" t="n"/>
+      <c r="B45" s="23" t="n"/>
+      <c r="C45" s="23" t="n"/>
+      <c r="D45" s="23" t="n"/>
+      <c r="E45" s="23" t="n"/>
+      <c r="F45" s="23" t="n"/>
+      <c r="G45" s="23" t="n"/>
+      <c r="H45" s="23" t="n"/>
+      <c r="I45" s="23" t="n"/>
+      <c r="J45" s="23" t="n"/>
+      <c r="K45" s="23" t="n"/>
+      <c r="L45" s="23" t="n"/>
+      <c r="M45" s="23" t="n"/>
+      <c r="N45" s="23" t="n"/>
+      <c r="O45" s="23" t="n"/>
+      <c r="P45" s="23" t="n"/>
+      <c r="Q45" s="23" t="n"/>
+      <c r="R45" s="23" t="n"/>
+      <c r="S45" s="9" t="n"/>
+    </row>
+    <row r="46" ht="15.6" customHeight="1" s="24">
+      <c r="A46" s="8" t="n"/>
+      <c r="B46" s="23" t="n"/>
+      <c r="C46" s="23" t="n"/>
+      <c r="D46" s="23" t="n"/>
+      <c r="E46" s="23" t="n"/>
+      <c r="F46" s="23" t="n"/>
+      <c r="G46" s="23" t="n"/>
+      <c r="H46" s="23" t="n"/>
+      <c r="I46" s="23" t="n"/>
+      <c r="J46" s="23" t="n"/>
+      <c r="K46" s="23" t="n"/>
+      <c r="L46" s="23" t="n"/>
+      <c r="M46" s="23" t="n"/>
+      <c r="N46" s="23" t="n"/>
+      <c r="O46" s="23" t="n"/>
+      <c r="P46" s="23" t="n"/>
+      <c r="Q46" s="23" t="n"/>
+      <c r="R46" s="23" t="n"/>
+      <c r="S46" s="9" t="n"/>
+    </row>
+    <row r="47" ht="15.6" customHeight="1" s="24">
+      <c r="A47" s="14" t="n"/>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>Elaboró</t>
+        </is>
+      </c>
+      <c r="C47" s="16" t="n"/>
+      <c r="D47" s="16" t="n"/>
+      <c r="E47" s="16" t="n"/>
+      <c r="F47" s="16" t="n"/>
+      <c r="G47" s="16" t="n"/>
+      <c r="H47" s="16" t="n"/>
+      <c r="I47" s="15" t="inlineStr">
+        <is>
+          <t>Revisó</t>
+        </is>
+      </c>
+      <c r="J47" s="16" t="n"/>
+      <c r="K47" s="16" t="n"/>
+      <c r="L47" s="16" t="n"/>
+      <c r="M47" s="16" t="n"/>
+      <c r="N47" s="16" t="n"/>
+      <c r="O47" s="16" t="n"/>
+      <c r="P47" s="15" t="inlineStr">
+        <is>
+          <t>Aprobó</t>
+        </is>
+      </c>
+      <c r="Q47" s="16" t="n"/>
+      <c r="R47" s="16" t="n"/>
+      <c r="S47" s="17" t="n"/>
+    </row>
+    <row r="48" ht="15.6" customHeight="1" s="24">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="23" t="n"/>
+      <c r="C48" s="23" t="n"/>
+      <c r="D48" s="23" t="n"/>
+      <c r="E48" s="23" t="n"/>
+      <c r="F48" s="23" t="n"/>
+      <c r="G48" s="23" t="n"/>
+      <c r="H48" s="23" t="n"/>
+      <c r="I48" s="23" t="n"/>
+      <c r="J48" s="23" t="n"/>
+      <c r="K48" s="23" t="n"/>
+      <c r="L48" s="23" t="n"/>
+      <c r="M48" s="23" t="n"/>
+      <c r="N48" s="23" t="n"/>
+      <c r="O48" s="23" t="n"/>
+      <c r="P48" s="23" t="n"/>
+      <c r="Q48" s="23" t="n"/>
+      <c r="R48" s="23" t="n"/>
+      <c r="S48" s="9" t="n"/>
+    </row>
+    <row r="49" ht="15.6" customHeight="1" s="24">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="23" t="n"/>
+      <c r="C49" s="23" t="n"/>
+      <c r="D49" s="23" t="n"/>
+      <c r="E49" s="23" t="n"/>
+      <c r="F49" s="23" t="n"/>
+      <c r="G49" s="23" t="n"/>
+      <c r="H49" s="23" t="n"/>
+      <c r="I49" s="23" t="n"/>
+      <c r="J49" s="23" t="n"/>
+      <c r="K49" s="23" t="n"/>
+      <c r="L49" s="23" t="n"/>
+      <c r="M49" s="23" t="n"/>
+      <c r="N49" s="23" t="n"/>
+      <c r="O49" s="23" t="n"/>
+      <c r="P49" s="23" t="n"/>
+      <c r="Q49" s="23" t="n"/>
+      <c r="R49" s="23" t="n"/>
+      <c r="S49" s="9" t="n"/>
+    </row>
+    <row r="50" ht="15.6" customHeight="1" s="24">
+      <c r="A50" s="8" t="n"/>
+      <c r="B50" s="11" t="n"/>
+      <c r="C50" s="11" t="n"/>
+      <c r="D50" s="11" t="n"/>
+      <c r="E50" s="23" t="n"/>
+      <c r="F50" s="23" t="n"/>
+      <c r="G50" s="23" t="n"/>
+      <c r="H50" s="23" t="n"/>
+      <c r="I50" s="11" t="n"/>
+      <c r="J50" s="11" t="n"/>
+      <c r="K50" s="11" t="n"/>
+      <c r="L50" s="23" t="n"/>
+      <c r="M50" s="23" t="n"/>
+      <c r="N50" s="23" t="n"/>
+      <c r="O50" s="23" t="n"/>
+      <c r="P50" s="11" t="n"/>
+      <c r="Q50" s="11" t="n"/>
+      <c r="R50" s="11" t="n"/>
+      <c r="S50" s="9" t="n"/>
+    </row>
+    <row r="51" ht="15.6" customHeight="1" s="24">
+      <c r="A51" s="8" t="n"/>
+      <c r="E51" s="23" t="n"/>
+      <c r="F51" s="23" t="n"/>
+      <c r="G51" s="23" t="n"/>
+      <c r="H51" s="23" t="n"/>
+      <c r="I51" s="38" t="n"/>
+      <c r="J51" s="27" t="n"/>
+      <c r="K51" s="27" t="n"/>
+      <c r="L51" s="23" t="n"/>
+      <c r="M51" s="23" t="n"/>
+      <c r="N51" s="23" t="n"/>
+      <c r="O51" s="23" t="n"/>
+      <c r="P51" s="38" t="n"/>
+      <c r="Q51" s="27" t="n"/>
+      <c r="R51" s="27" t="n"/>
+      <c r="S51" s="9" t="n"/>
+    </row>
+    <row r="52" ht="15.6" customHeight="1" s="24">
+      <c r="A52" s="8" t="n"/>
+      <c r="E52" s="23" t="n"/>
+      <c r="F52" s="23" t="n"/>
+      <c r="G52" s="23" t="n"/>
+      <c r="H52" s="23" t="n"/>
+      <c r="I52" s="23" t="n"/>
+      <c r="L52" s="23" t="n"/>
+      <c r="M52" s="23" t="n"/>
+      <c r="N52" s="23" t="n"/>
+      <c r="O52" s="23" t="n"/>
+      <c r="P52" s="23" t="n"/>
+      <c r="S52" s="9" t="n"/>
+    </row>
+    <row r="53" ht="15.6" customHeight="1" s="24">
+      <c r="A53" s="8" t="n"/>
+      <c r="E53" s="23" t="n"/>
+      <c r="F53" s="23" t="n"/>
+      <c r="G53" s="23" t="n"/>
+      <c r="H53" s="23" t="n"/>
+      <c r="I53" s="36" t="n"/>
+      <c r="L53" s="23" t="n"/>
+      <c r="M53" s="23" t="n"/>
+      <c r="N53" s="23" t="n"/>
+      <c r="O53" s="23" t="n"/>
+      <c r="P53" s="36" t="n"/>
+      <c r="S53" s="9" t="n"/>
+    </row>
+    <row r="54" ht="15.6" customHeight="1" s="24">
+      <c r="A54" s="8" t="n"/>
+      <c r="B54" s="23" t="n"/>
+      <c r="C54" s="23" t="n"/>
+      <c r="D54" s="23" t="n"/>
+      <c r="E54" s="23" t="n"/>
+      <c r="F54" s="23" t="n"/>
+      <c r="G54" s="23" t="n"/>
+      <c r="H54" s="23" t="n"/>
+      <c r="I54" s="23" t="n"/>
+      <c r="J54" s="23" t="n"/>
+      <c r="K54" s="23" t="n"/>
+      <c r="L54" s="23" t="n"/>
+      <c r="M54" s="23" t="n"/>
+      <c r="N54" s="23" t="n"/>
+      <c r="O54" s="23" t="n"/>
+      <c r="P54" s="23" t="n"/>
+      <c r="Q54" s="23" t="n"/>
+      <c r="R54" s="23" t="n"/>
+      <c r="S54" s="9" t="n"/>
+    </row>
+    <row r="55" ht="15.6" customHeight="1" s="24">
+      <c r="A55" s="10" t="n"/>
+      <c r="B55" s="11" t="n"/>
+      <c r="C55" s="11" t="n"/>
+      <c r="D55" s="11" t="n"/>
+      <c r="E55" s="11" t="n"/>
+      <c r="F55" s="11" t="n"/>
+      <c r="G55" s="11" t="n"/>
+      <c r="H55" s="11" t="n"/>
+      <c r="I55" s="11" t="n"/>
+      <c r="J55" s="11" t="n"/>
+      <c r="K55" s="11" t="n"/>
+      <c r="L55" s="11" t="n"/>
+      <c r="M55" s="11" t="n"/>
+      <c r="N55" s="11" t="n"/>
+      <c r="O55" s="11" t="n"/>
+      <c r="P55" s="11" t="n"/>
+      <c r="Q55" s="11" t="n"/>
+      <c r="R55" s="11" t="n"/>
+      <c r="S55" s="12" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="51">
+    <mergeCell ref="B40:R44"/>
+    <mergeCell ref="P52:R52"/>
+    <mergeCell ref="K32:M32"/>
+    <mergeCell ref="D12:M12"/>
+    <mergeCell ref="K22:M22"/>
+    <mergeCell ref="E3:O7"/>
+    <mergeCell ref="I53:K53"/>
+    <mergeCell ref="K31:M31"/>
+    <mergeCell ref="R15:R16"/>
+    <mergeCell ref="B16:J37"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="K15:M16"/>
+    <mergeCell ref="K37:Q37"/>
+    <mergeCell ref="E8:O10"/>
+    <mergeCell ref="N12:O12"/>
+    <mergeCell ref="I52:K52"/>
+    <mergeCell ref="K27:M27"/>
+    <mergeCell ref="B39:R39"/>
+    <mergeCell ref="D13:H13"/>
+    <mergeCell ref="K23:M23"/>
+    <mergeCell ref="P53:R53"/>
+    <mergeCell ref="B11:R11"/>
+    <mergeCell ref="K17:M17"/>
+    <mergeCell ref="P12:R12"/>
+    <mergeCell ref="Q15:Q16"/>
+    <mergeCell ref="P3:R3"/>
+    <mergeCell ref="I51:K51"/>
+    <mergeCell ref="B14:R14"/>
+    <mergeCell ref="B15:J15"/>
+    <mergeCell ref="N15:P15"/>
+    <mergeCell ref="K19:M19"/>
+    <mergeCell ref="B3:D10"/>
+    <mergeCell ref="K28:M28"/>
+    <mergeCell ref="P5:R5"/>
+    <mergeCell ref="K13:P13"/>
+    <mergeCell ref="K18:M18"/>
+    <mergeCell ref="K34:M34"/>
+    <mergeCell ref="P4:R4"/>
+    <mergeCell ref="P51:R51"/>
+    <mergeCell ref="K30:M30"/>
+    <mergeCell ref="K25:M25"/>
+    <mergeCell ref="K33:M33"/>
+    <mergeCell ref="K24:M24"/>
+    <mergeCell ref="P9:Q10"/>
+    <mergeCell ref="K36:M36"/>
+    <mergeCell ref="K20:M20"/>
+    <mergeCell ref="K21:M21"/>
     <mergeCell ref="K35:M35"/>
     <mergeCell ref="K26:M26"/>
     <mergeCell ref="K29:M29"/>
@@ -15777,7 +18065,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Excavacion masiva plataforma</t>
+          <t>Excavacion masiva plataforma (reemplazo bajo placa)</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -15786,7 +18074,7 @@
         <v>9.85</v>
       </c>
       <c r="O17" s="18" t="n">
-        <v>0.55</v>
+        <v>0.6</v>
       </c>
       <c r="P17" s="18" t="n">
         <v>21.95</v>
@@ -16144,7 +18432,7 @@
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>VERIFICAR EN DWG: la huella 9.85 x 21.95 no esta acotada en los PDF. La reticula estructural acotada es 19.80 (ejes 1-4) x 7.30/7.70 (ejes A-B). Confirmar la dimension en el plano arquitectonico/DWG y pegar el pantallazo.</t>
+          <t>CORREGIDO: prof. 0.60 m = recebo 0.20 + sub-base 0.30 + placa 0.10 (paquete de reemplazo bajo la placa, hasta nivel -0.65). Antes 0.55 no cuadraba. Huella 9.85x21.95 sigue pendiente de confirmar en DWG.</t>
         </is>
       </c>
       <c r="C40" s="27" t="n"/>
@@ -16887,7 +19175,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Capa subbase bajo placa e=0.15</t>
+          <t>Capa sub-base bajo placa e=0.30</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -16896,7 +19184,7 @@
         <v>9.85</v>
       </c>
       <c r="O17" s="18" t="n">
-        <v>0.15</v>
+        <v>0.3</v>
       </c>
       <c r="P17" s="18" t="n">
         <v>21.95</v>
@@ -17254,7 +19542,7 @@
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>VERIFICAR EN DWG: la huella 9.85 x 21.95 no esta acotada en los PDF. La reticula estructural acotada es 19.80 (ejes 1-4) x 7.30/7.70 (ejes A-B). Confirmar la dimension en el plano arquitectonico/DWG y pegar el pantallazo.</t>
+          <t>CORREGIDO: e=0.30 m. El detalle de losa de contrapiso dice 'SUB-BASE DE 30 cm' y 'Minimo 0.30m'. Antes estaba en 0.15.</t>
         </is>
       </c>
       <c r="C40" s="27" t="n"/>
@@ -17997,7 +20285,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Zanjas vigas long. A,B</t>
+          <t>Zanjas vigas long. A,B (0.40x0.45, de -0.65 a -1.10)</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -18006,7 +20294,7 @@
         <v>0.4</v>
       </c>
       <c r="O17" s="18" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="P17" s="18" t="n">
         <v>19.8</v>
@@ -18026,7 +20314,7 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Zanjas vigas transv. (luz libre)</t>
+          <t>Zanjas vigas transv. (0.40x0.45)</t>
         </is>
       </c>
       <c r="L18" s="21" t="n"/>
@@ -18035,7 +20323,7 @@
         <v>0.4</v>
       </c>
       <c r="O18" s="18" t="n">
-        <v>0.4</v>
+        <v>0.45</v>
       </c>
       <c r="P18" s="18" t="n">
         <v>7.3</v>
@@ -18053,28 +20341,58 @@
       <c r="A19" s="8" t="n"/>
       <c r="B19" s="29" t="n"/>
       <c r="J19" s="30" t="n"/>
-      <c r="K19" s="20" t="n"/>
+      <c r="K19" s="20" t="inlineStr">
+        <is>
+          <t>Fosos zapatas Z-1 (2.30x2.30) prof 0.90 (de -0.65 a -1.55)</t>
+        </is>
+      </c>
       <c r="L19" s="21" t="n"/>
       <c r="M19" s="22" t="n"/>
-      <c r="N19" s="18" t="n"/>
-      <c r="O19" s="18" t="n"/>
-      <c r="P19" s="18" t="n"/>
-      <c r="Q19" s="18" t="n"/>
-      <c r="R19" s="18" t="n"/>
+      <c r="N19" s="18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="O19" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="P19" s="18" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="Q19" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R19" s="18">
+        <f>N19*O19*P19*Q19</f>
+        <v/>
+      </c>
       <c r="S19" s="9" t="n"/>
     </row>
     <row r="20" ht="15.6" customHeight="1" s="24">
       <c r="A20" s="8" t="n"/>
       <c r="B20" s="29" t="n"/>
       <c r="J20" s="30" t="n"/>
-      <c r="K20" s="20" t="n"/>
+      <c r="K20" s="20" t="inlineStr">
+        <is>
+          <t>Fosos zapatas Z-2 (2.15x2.15) prof 0.90</t>
+        </is>
+      </c>
       <c r="L20" s="21" t="n"/>
       <c r="M20" s="22" t="n"/>
-      <c r="N20" s="18" t="n"/>
-      <c r="O20" s="18" t="n"/>
-      <c r="P20" s="18" t="n"/>
-      <c r="Q20" s="18" t="n"/>
-      <c r="R20" s="18" t="n"/>
+      <c r="N20" s="18" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="O20" s="18" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="P20" s="18" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="Q20" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="R20" s="18">
+        <f>N20*O20*P20*Q20</f>
+        <v/>
+      </c>
       <c r="S20" s="9" t="n"/>
     </row>
     <row r="21" ht="15.6" customHeight="1" s="24">
@@ -18377,7 +20695,11 @@
     </row>
     <row r="40" ht="15.6" customHeight="1" s="24">
       <c r="A40" s="8" t="n"/>
-      <c r="B40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>CORREGIDO: excavacion manual por debajo del nivel masivo (-0.65): zanjas de vigas 0.45 m de prof (altura de la viga) + fosos de zapatas 0.90 m hasta el desplante (-1.55). Estimacion sin descontar solapes viga-zapata (conservador).</t>
+        </is>
+      </c>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="27" t="n"/>
       <c r="E40" s="27" t="n"/>

</xml_diff>

<commit_message>
fix(columnas): alturas 4.75/4.95 (de -0.05 a +4.70/+4.90), volumen 7.99 m3
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
@@ -3397,7 +3397,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Columnas tipo 1 (0.40x0.40) h=4.70 - ejes 1A,1B,3'B,4A</t>
+          <t>Columnas tipo 1 (0.40x0.40) h=4.75 - ejes 1A,1B,3'B,4A</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -3409,7 +3409,7 @@
         <v>0.4</v>
       </c>
       <c r="P17" s="18" t="n">
-        <v>4.7</v>
+        <v>4.75</v>
       </c>
       <c r="Q17" s="18" t="n">
         <v>4</v>
@@ -3426,7 +3426,7 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Columnas tipo 2 (0.50x0.50) h=4.90 - ejes 2A,2B,3A,3B</t>
+          <t>Columnas tipo 2 (0.50x0.50) h=4.95 - ejes 2A,2B,3A,3B</t>
         </is>
       </c>
       <c r="L18" s="21" t="n"/>
@@ -3438,7 +3438,7 @@
         <v>0.5</v>
       </c>
       <c r="P18" s="18" t="n">
-        <v>4.9</v>
+        <v>4.95</v>
       </c>
       <c r="Q18" s="18" t="n">
         <v>4</v>
@@ -3779,7 +3779,7 @@
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>CORREGIDO: el despiece de columnas muestra 8 columnas en 2 tipos (4 de 0.40x0.40 y 4 de 0.50x0.50). Antes se habia puesto 10 col de 0.40x0.40.</t>
+          <t>CORREGIDO: 8 columnas en 2 tipos. Alturas de -0.05 a +4.70 (T1=4.75) y a +4.90 (T2=4.95), leidas de los niveles del despiece. Vol total = 7.99 m3.</t>
         </is>
       </c>
       <c r="C40" s="27" t="n"/>

</xml_diff>

<commit_message>
fix(2.1.1): excavacion masiva = 0.40 m (sub-base+placa); el recebo va aparte, no se suma
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
@@ -18065,7 +18065,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Excavacion masiva plataforma (reemplazo bajo placa)</t>
+          <t>Excavacion masiva plataforma (sub-base 0.30 + placa 0.10)</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -18074,7 +18074,7 @@
         <v>9.85</v>
       </c>
       <c r="O17" s="18" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="P17" s="18" t="n">
         <v>21.95</v>
@@ -18432,7 +18432,7 @@
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>CORREGIDO: prof. 0.60 m = recebo 0.20 + sub-base 0.30 + placa 0.10 (paquete de reemplazo bajo la placa, hasta nivel -0.65). Antes 0.55 no cuadraba. Huella 9.85x21.95 sigue pendiente de confirmar en DWG.</t>
+          <t>CORREGIDO: 0.60 -&gt; 0.40 m. El detalle de la losa solo muestra sub-base 0.30 + placa 0.10. El recebo (2.1.4) NO va aqui: es relleno que va en otra parte (backfill sobre las vigas). Huella 9.85x21.95 aun por confirmar en DWG.</t>
         </is>
       </c>
       <c r="C40" s="27" t="n"/>

</xml_diff>

<commit_message>
chore: limpiar valores residuales (N/O/P) en hojas de acero de la memoria
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
@@ -8989,15 +8989,9 @@
       </c>
       <c r="L17" s="21" t="n"/>
       <c r="M17" s="22" t="n"/>
-      <c r="N17" s="18" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="O17" s="18" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="P17" s="18" t="n">
-        <v>21.95</v>
-      </c>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
+      <c r="P17" s="18" t="n"/>
       <c r="Q17" s="18" t="n">
         <v>1</v>
       </c>
@@ -10112,15 +10106,9 @@
       </c>
       <c r="L17" s="21" t="n"/>
       <c r="M17" s="22" t="n"/>
-      <c r="N17" s="18" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="O17" s="18" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="P17" s="18" t="n">
-        <v>21.95</v>
-      </c>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
+      <c r="P17" s="18" t="n"/>
       <c r="Q17" s="18" t="n">
         <v>1</v>
       </c>
@@ -11239,15 +11227,9 @@
       </c>
       <c r="L17" s="21" t="n"/>
       <c r="M17" s="22" t="n"/>
-      <c r="N17" s="18" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="O17" s="18" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="P17" s="18" t="n">
-        <v>21.95</v>
-      </c>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
+      <c r="P17" s="18" t="n"/>
       <c r="Q17" s="18" t="n">
         <v>1</v>
       </c>
@@ -12362,15 +12344,9 @@
       </c>
       <c r="L17" s="21" t="n"/>
       <c r="M17" s="22" t="n"/>
-      <c r="N17" s="18" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="O17" s="18" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="P17" s="18" t="n">
-        <v>21.95</v>
-      </c>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
+      <c r="P17" s="18" t="n"/>
       <c r="Q17" s="18" t="n">
         <v>1</v>
       </c>
@@ -15745,15 +15721,9 @@
       </c>
       <c r="L17" s="21" t="n"/>
       <c r="M17" s="22" t="n"/>
-      <c r="N17" s="18" t="n">
-        <v>9.85</v>
-      </c>
-      <c r="O17" s="18" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="P17" s="18" t="n">
-        <v>21.95</v>
-      </c>
+      <c r="N17" s="18" t="n"/>
+      <c r="O17" s="18" t="n"/>
+      <c r="P17" s="18" t="n"/>
       <c r="Q17" s="18" t="n">
         <v>1</v>
       </c>

</xml_diff>

<commit_message>
Recalcular acero por peso con tabla de masas de varilla
- Metodo: L(m) por calibre x masa (kg/m) + 10%, barras de los despieces
- 4.7.1 columnas: 1367.6 kg (6#6 T1; 4#6+4#7 T2; estribos+grapas #3)
- 2.3.1 vigas cim: 1401.9 kg (VC-1..4,3',A,B; estribos #3 L=1.58)
- 4.8.1 vigas cubierta: 1593.8 kg (VG-1..4 + VG-6/7; estribos #3 L=1.68)
- 2.3.2 zapatas: 652.8 kg (#5@0.20 dos sentidos)
- 5.2.1 mamposteria: 374.6 kg (columneta 2#4+est#3; cinta 2#3+gancho#2)
- Word: seccion de metodo de acero + tabla de masas + items actualizados
</commit_message>
<xml_diff>
--- a/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
+++ b/Proyectos/Fundamentos-de-Construccion/MEMORIAS DE CALCULO.xlsx
@@ -8984,7 +8984,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Long. 3#6+3#5 (kg)</t>
+          <t>Long. #6 (236.7 m) + #5 (276.2 m) - VC-1..4,3',A,B</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -8996,7 +8996,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="18" t="n">
-        <v>864.6</v>
+        <v>957.7</v>
       </c>
       <c r="S17" s="9" t="n"/>
     </row>
@@ -9006,7 +9006,7 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Estribos #3 c/0.20 (kg)</t>
+          <t>Estribos #3 L=1.58 (5x36 transv + 2x89 long)</t>
         </is>
       </c>
       <c r="L18" s="21" t="n"/>
@@ -9016,7 +9016,7 @@
       <c r="P18" s="18" t="n"/>
       <c r="Q18" s="18" t="n"/>
       <c r="R18" s="18" t="n">
-        <v>319.6</v>
+        <v>316.8</v>
       </c>
       <c r="S18" s="9" t="n"/>
     </row>
@@ -9036,7 +9036,7 @@
       <c r="P19" s="18" t="n"/>
       <c r="Q19" s="18" t="n"/>
       <c r="R19" s="18" t="n">
-        <v>1184.2</v>
+        <v>1274.5</v>
       </c>
       <c r="S19" s="9" t="n"/>
     </row>
@@ -9056,7 +9056,7 @@
       <c r="P20" s="18" t="n"/>
       <c r="Q20" s="18" t="n"/>
       <c r="R20" s="18" t="n">
-        <v>1302.6</v>
+        <v>1402</v>
       </c>
       <c r="S20" s="9" t="n"/>
     </row>
@@ -9360,7 +9360,11 @@
     </row>
     <row r="40" ht="15.6" customHeight="1" s="24">
       <c r="A40" s="8" t="n"/>
-      <c r="B40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>Por peso con tabla de masas: #5=1.552, #6=2.235, #3=0.560 kg/m; +10%. Barras del despiece: VC-1/2/3/3'/4 (transv) y VC-A/VC-B (long). VC-3 se asume = VC-2.</t>
+        </is>
+      </c>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="27" t="n"/>
       <c r="E40" s="27" t="n"/>
@@ -10101,7 +10105,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Long. Tipo1 (4col x 6#6 L=5.85) + Tipo2 (4col x 4#6+4#7 L=5.95)</t>
+          <t>Long. #6+#7 (T1:6#6 L5.85 / T2:4#6+4#7 L5.95) x8 col</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -10113,7 +10117,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="18" t="n">
-        <v>628</v>
+        <v>816.2</v>
       </c>
       <c r="S17" s="9" t="n"/>
     </row>
@@ -10123,7 +10127,7 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Estribos #2 c/0.20 (kg)</t>
+          <t>Estribos+grapas #3 (T1:42x1.48+42x0.54 / T2:42x1.88+42x0.64) x8</t>
         </is>
       </c>
       <c r="L18" s="21" t="n"/>
@@ -10133,7 +10137,7 @@
       <c r="P18" s="18" t="n"/>
       <c r="Q18" s="18" t="n"/>
       <c r="R18" s="18" t="n">
-        <v>91.90000000000001</v>
+        <v>427.1</v>
       </c>
       <c r="S18" s="9" t="n"/>
     </row>
@@ -10153,7 +10157,7 @@
       <c r="P19" s="18" t="n"/>
       <c r="Q19" s="18" t="n"/>
       <c r="R19" s="18" t="n">
-        <v>719.8</v>
+        <v>1243.3</v>
       </c>
       <c r="S19" s="9" t="n"/>
     </row>
@@ -10173,7 +10177,7 @@
       <c r="P20" s="18" t="n"/>
       <c r="Q20" s="18" t="n"/>
       <c r="R20" s="18" t="n">
-        <v>791.8</v>
+        <v>1367.6</v>
       </c>
       <c r="S20" s="9" t="n"/>
     </row>
@@ -10479,7 +10483,7 @@
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>REVISAR: el refuerzo longitudinal difiere por tipo de columna (Tipo1: 6#6; Tipo2: 4#6+4#7). El peso exacto (kg) debe salir de la cartilla de hierros (DLNET). El valor mostrado es una estimacion con +10%.</t>
+          <t>Calculado por peso con tabla de masas de varilla: L(m)xkg/m + 10%. kg/m usados: #3=0.560, #6=2.235, #7=3.042. Barras del despiece de columnas (Son 4 c/tipo).</t>
         </is>
       </c>
       <c r="C40" s="27" t="n"/>
@@ -11222,7 +11226,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Long. 2#6+2#7+2#6 (kg)</t>
+          <t>Long. #5 (252.8 m) + #6 (196.6 m) - VG-1..4 + VG-6/VG-7</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -11234,7 +11238,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="18" t="n">
-        <v>1143.3</v>
+        <v>831.7</v>
       </c>
       <c r="S17" s="9" t="n"/>
     </row>
@@ -11244,7 +11248,7 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Estribos #3 c/0.15 (kg)</t>
+          <t>Estribos #3 L=1.68 (4x73 transv + 2x182 long)</t>
         </is>
       </c>
       <c r="L18" s="21" t="n"/>
@@ -11254,7 +11258,7 @@
       <c r="P18" s="18" t="n"/>
       <c r="Q18" s="18" t="n"/>
       <c r="R18" s="18" t="n">
-        <v>454.6</v>
+        <v>617.2</v>
       </c>
       <c r="S18" s="9" t="n"/>
     </row>
@@ -11274,7 +11278,7 @@
       <c r="P19" s="18" t="n"/>
       <c r="Q19" s="18" t="n"/>
       <c r="R19" s="18" t="n">
-        <v>1597.9</v>
+        <v>1448.9</v>
       </c>
       <c r="S19" s="9" t="n"/>
     </row>
@@ -11294,7 +11298,7 @@
       <c r="P20" s="18" t="n"/>
       <c r="Q20" s="18" t="n"/>
       <c r="R20" s="18" t="n">
-        <v>1757.7</v>
+        <v>1593.8</v>
       </c>
       <c r="S20" s="9" t="n"/>
     </row>
@@ -11598,7 +11602,11 @@
     </row>
     <row r="40" ht="15.6" customHeight="1" s="24">
       <c r="A40" s="8" t="n"/>
-      <c r="B40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>Por peso con tabla de masas: #5=1.552, #6=2.235, #3=0.560 kg/m; +10%. NO incluye viguetas (placa aligerada): 6 viguetas 0.20x0.40 con #4 y est.#3 = 1689.1 kg aprox, contabilizar en la placa de cubierta si aplica.</t>
+        </is>
+      </c>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="27" t="n"/>
       <c r="E40" s="27" t="n"/>
@@ -12339,7 +12347,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Long. 4#3 (kg)</t>
+          <t>Columnetas 2#4 (0.20x0.15) + Cinta V2 2#3</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -12351,7 +12359,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="18" t="n">
-        <v>376.8</v>
+        <v>207.2</v>
       </c>
       <c r="S17" s="9" t="n"/>
     </row>
@@ -12361,7 +12369,7 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Estribos #2 c/0.20 (kg)</t>
+          <t>Estribo #3 c/0.20 (columneta) + gancho #2 (1/4") c/0.30 (cinta)</t>
         </is>
       </c>
       <c r="L18" s="21" t="n"/>
@@ -12371,7 +12379,7 @@
       <c r="P18" s="18" t="n"/>
       <c r="Q18" s="18" t="n"/>
       <c r="R18" s="18" t="n">
-        <v>105.1</v>
+        <v>133.3</v>
       </c>
       <c r="S18" s="9" t="n"/>
     </row>
@@ -12391,7 +12399,7 @@
       <c r="P19" s="18" t="n"/>
       <c r="Q19" s="18" t="n"/>
       <c r="R19" s="18" t="n">
-        <v>481.9</v>
+        <v>340.5</v>
       </c>
       <c r="S19" s="9" t="n"/>
     </row>
@@ -12411,7 +12419,7 @@
       <c r="P20" s="18" t="n"/>
       <c r="Q20" s="18" t="n"/>
       <c r="R20" s="18" t="n">
-        <v>530.1</v>
+        <v>374.6</v>
       </c>
       <c r="S20" s="9" t="n"/>
     </row>
@@ -12715,7 +12723,11 @@
     </row>
     <row r="40" ht="15.6" customHeight="1" s="24">
       <c r="A40" s="8" t="n"/>
-      <c r="B40" s="20" t="n"/>
+      <c r="B40" s="20" t="inlineStr">
+        <is>
+          <t>ESTIMACION por peso (tabla masas): columneta 2#4+est#3; cinta V2 2#3+gancho#2. Cantidades (24 columnetas h=2.70; 70 m de cinta) POR CONFIRMAR en el plano de mamposteria FC3.</t>
+        </is>
+      </c>
       <c r="C40" s="27" t="n"/>
       <c r="D40" s="27" t="n"/>
       <c r="E40" s="27" t="n"/>
@@ -15716,7 +15728,7 @@
       <c r="J17" s="30" t="n"/>
       <c r="K17" s="20" t="inlineStr">
         <is>
-          <t>Z-1: 4 zap, #5@0.20 dos sentidos (est.)</t>
+          <t>Z-1 (4) 2.30x2.30  #5@0.20 dos sentidos</t>
         </is>
       </c>
       <c r="L17" s="21" t="n"/>
@@ -15728,7 +15740,7 @@
         <v>1</v>
       </c>
       <c r="R17" s="18" t="n">
-        <v>327.8</v>
+        <v>320.3</v>
       </c>
       <c r="S17" s="9" t="n"/>
     </row>
@@ -15738,7 +15750,7 @@
       <c r="J18" s="30" t="n"/>
       <c r="K18" s="20" t="inlineStr">
         <is>
-          <t>Z-2: 4 zap, #5@0.20 dos sentidos (est.)</t>
+          <t>Z-2 (4) 2.15x2.15  #5@0.20 dos sentidos</t>
         </is>
       </c>
       <c r="L18" s="21" t="n"/>
@@ -15748,7 +15760,7 @@
       <c r="P18" s="18" t="n"/>
       <c r="Q18" s="18" t="n"/>
       <c r="R18" s="18" t="n">
-        <v>280</v>
+        <v>273.2</v>
       </c>
       <c r="S18" s="9" t="n"/>
     </row>
@@ -15768,7 +15780,7 @@
       <c r="P19" s="18" t="n"/>
       <c r="Q19" s="18" t="n"/>
       <c r="R19" s="18" t="n">
-        <v>607.8</v>
+        <v>593.5</v>
       </c>
       <c r="S19" s="9" t="n"/>
     </row>
@@ -15788,7 +15800,7 @@
       <c r="P20" s="18" t="n"/>
       <c r="Q20" s="18" t="n"/>
       <c r="R20" s="18" t="n">
-        <v>668.6</v>
+        <v>652.9</v>
       </c>
       <c r="S20" s="9" t="n"/>
     </row>
@@ -16094,7 +16106,7 @@
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="20" t="inlineStr">
         <is>
-          <t>AGREGADO (ESTIMACION): #5 @0.20 en ambos sentidos, ambas zapatas. El peso exacto debe salir de la cartilla de hierros (DLNET). Falta linea en el presupuesto.</t>
+          <t>Por peso con tabla de masas: #5=1.552 kg/m; +10%. Lbarra=lado-0.15 (recubr.); n=lado/0.20+1 por sentido. Confirmar lados exactos en DWG.</t>
         </is>
       </c>
       <c r="C40" s="27" t="n"/>

</xml_diff>